<commit_message>
ID format T/L/P-0001, no reuse of deleted IDs, ID validation in v6
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -1779,16 +1779,20 @@
           <t>ID закрыть</t>
         </is>
       </c>
-      <c r="H10" s="194" t="n">
-        <v>1</v>
+      <c r="H10" s="194" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
           <t>ID закрыть</t>
         </is>
       </c>
-      <c r="J10" s="194" t="n">
-        <v>1</v>
+      <c r="J10" s="194" t="inlineStr">
+        <is>
+          <t>L-0001</t>
+        </is>
       </c>
       <c r="K10" s="207" t="n"/>
       <c r="L10" s="207" t="n"/>
@@ -1891,8 +1895,10 @@
           <t>ID позиции</t>
         </is>
       </c>
-      <c r="H15" s="194" t="n">
-        <v>1</v>
+      <c r="H15" s="194" t="inlineStr">
+        <is>
+          <t>P-0001</t>
+        </is>
       </c>
       <c r="I15" s="14" t="inlineStr">
         <is>
@@ -2060,7 +2066,7 @@
     <mergeCell ref="B1:J2"/>
     <mergeCell ref="G3:J3"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="11">
     <dataValidation sqref="H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Добавить,Удалить"</formula1>
     </dataValidation>
@@ -2085,6 +2091,15 @@
     </dataValidation>
     <dataValidation sqref="H7 H8" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Число" error="Введите число больше нуля." type="decimal" operator="greaterThan">
       <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ID закрыть" error="Формат ID: T-0001 (буква T, дефис и номер минимум из четырёх цифр)." type="custom">
+      <formula1>=IFERROR(AND(EXACT(LEFT(H10,2),"T-"),ISNUMBER(--MID(H10,3,20)),MID(H10,3,20)=TEXT(--MID(H10,3,20),"0000")),FALSE)</formula1>
+    </dataValidation>
+    <dataValidation sqref="J10" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ID закрыть" error="Формат ID: L-0001 (буква L, дефис и номер минимум из четырёх цифр)." type="custom">
+      <formula1>=IFERROR(AND(EXACT(LEFT(J10,2),"L-"),ISNUMBER(--MID(J10,3,20)),MID(J10,3,20)=TEXT(--MID(J10,3,20),"0000")),FALSE)</formula1>
+    </dataValidation>
+    <dataValidation sqref="H15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ID позиции" error="Формат ID: P-0001 (буква P, дефис и номер минимум из четырёх цифр)." type="custom">
+      <formula1>=IFERROR(AND(EXACT(LEFT(H15,2),"P-"),ISNUMBER(--MID(H15,3,20)),MID(H15,3,20)=TEXT(--MID(H15,3,20),"0000")),FALSE)</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
v6: demo IDs in journal sheets converted to T/L/P-0001
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -2313,8 +2313,10 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="186" t="n">
-        <v>1</v>
+      <c r="B5" s="186" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
       </c>
       <c r="C5" s="209" t="n">
         <v>46296</v>
@@ -2355,8 +2357,10 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="187" t="n">
-        <v>2</v>
+      <c r="B6" s="187" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
       </c>
       <c r="C6" s="210" t="n">
         <v>46296</v>
@@ -2397,8 +2401,10 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="n">
-        <v>3</v>
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
       </c>
       <c r="C7" s="209" t="n">
         <v>46297</v>
@@ -2439,8 +2445,10 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="n">
-        <v>4</v>
+      <c r="B8" s="187" t="inlineStr">
+        <is>
+          <t>T-0004</t>
+        </is>
       </c>
       <c r="C8" s="210" t="n">
         <v>46298</v>
@@ -2481,8 +2489,10 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="186" t="n">
-        <v>5</v>
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>T-0005</t>
+        </is>
       </c>
       <c r="C9" s="209" t="n">
         <v>46298</v>
@@ -2523,8 +2533,10 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="187" t="n">
-        <v>6</v>
+      <c r="B10" s="187" t="inlineStr">
+        <is>
+          <t>T-0006</t>
+        </is>
       </c>
       <c r="C10" s="210" t="n">
         <v>46299</v>
@@ -2565,8 +2577,10 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="n">
-        <v>7</v>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>T-0007</t>
+        </is>
       </c>
       <c r="C11" s="209" t="n">
         <v>46299</v>
@@ -2607,8 +2621,10 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="n">
-        <v>8</v>
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>T-0008</t>
+        </is>
       </c>
       <c r="C12" s="210" t="n">
         <v>46299</v>
@@ -3181,8 +3197,10 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="186" t="n">
-        <v>1</v>
+      <c r="B5" s="186" t="inlineStr">
+        <is>
+          <t>L-0001</t>
+        </is>
       </c>
       <c r="C5" s="209" t="n">
         <v>46296</v>
@@ -3223,8 +3241,10 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="187" t="n">
-        <v>2</v>
+      <c r="B6" s="187" t="inlineStr">
+        <is>
+          <t>L-0002</t>
+        </is>
       </c>
       <c r="C6" s="210" t="n">
         <v>46296</v>
@@ -3265,8 +3285,10 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="n">
-        <v>3</v>
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>L-0003</t>
+        </is>
       </c>
       <c r="C7" s="209" t="n">
         <v>46297</v>
@@ -3307,8 +3329,10 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="n">
-        <v>4</v>
+      <c r="B8" s="187" t="inlineStr">
+        <is>
+          <t>L-0004</t>
+        </is>
       </c>
       <c r="C8" s="210" t="n">
         <v>46298</v>
@@ -3349,8 +3373,10 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="186" t="n">
-        <v>5</v>
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>L-0005</t>
+        </is>
       </c>
       <c r="C9" s="209" t="n">
         <v>46298</v>
@@ -3391,8 +3417,10 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="187" t="n">
-        <v>6</v>
+      <c r="B10" s="187" t="inlineStr">
+        <is>
+          <t>L-0006</t>
+        </is>
       </c>
       <c r="C10" s="210" t="n">
         <v>46299</v>
@@ -3433,8 +3461,10 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="n">
-        <v>7</v>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>L-0007</t>
+        </is>
       </c>
       <c r="C11" s="209" t="n">
         <v>46299</v>
@@ -3475,8 +3505,10 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="n">
-        <v>8</v>
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>L-0008</t>
+        </is>
       </c>
       <c r="C12" s="210" t="n">
         <v>46299</v>
@@ -4013,8 +4045,10 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="186" t="n">
-        <v>1</v>
+      <c r="B5" s="186" t="inlineStr">
+        <is>
+          <t>P-0001</t>
+        </is>
       </c>
       <c r="C5" s="209" t="n">
         <v>46296</v>
@@ -4037,8 +4071,10 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="187" t="n">
-        <v>2</v>
+      <c r="B6" s="187" t="inlineStr">
+        <is>
+          <t>P-0002</t>
+        </is>
       </c>
       <c r="C6" s="210" t="n">
         <v>46296</v>
@@ -4061,8 +4097,10 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="n">
-        <v>3</v>
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>P-0003</t>
+        </is>
       </c>
       <c r="C7" s="209" t="n">
         <v>46297</v>
@@ -4085,8 +4123,10 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="n">
-        <v>4</v>
+      <c r="B8" s="187" t="inlineStr">
+        <is>
+          <t>P-0004</t>
+        </is>
       </c>
       <c r="C8" s="210" t="n">
         <v>46298</v>
@@ -4109,8 +4149,10 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="186" t="n">
-        <v>5</v>
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>P-0005</t>
+        </is>
       </c>
       <c r="C9" s="209" t="n">
         <v>46298</v>
@@ -4133,8 +4175,10 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="187" t="n">
-        <v>6</v>
+      <c r="B10" s="187" t="inlineStr">
+        <is>
+          <t>P-0006</t>
+        </is>
       </c>
       <c r="C10" s="210" t="n">
         <v>46299</v>
@@ -4157,8 +4201,10 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="n">
-        <v>7</v>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>P-0007</t>
+        </is>
       </c>
       <c r="C11" s="209" t="n">
         <v>46299</v>
@@ -4181,8 +4227,10 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="n">
-        <v>8</v>
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>P-0008</t>
+        </is>
       </c>
       <c r="C12" s="210" t="n">
         <v>46299</v>
@@ -4747,8 +4795,10 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="186" t="n">
-        <v>1</v>
+      <c r="B5" s="186" t="inlineStr">
+        <is>
+          <t>T-0001</t>
+        </is>
       </c>
       <c r="C5" s="209" t="n">
         <v>46296</v>
@@ -4801,8 +4851,10 @@
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="187" t="n">
-        <v>2</v>
+      <c r="B6" s="187" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
       </c>
       <c r="C6" s="210" t="n">
         <v>46296</v>
@@ -4855,8 +4907,10 @@
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="n">
-        <v>3</v>
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
       </c>
       <c r="C7" s="209" t="n">
         <v>46297</v>
@@ -4909,8 +4963,10 @@
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="n">
-        <v>4</v>
+      <c r="B8" s="187" t="inlineStr">
+        <is>
+          <t>T-0004</t>
+        </is>
       </c>
       <c r="C8" s="210" t="n">
         <v>46298</v>
@@ -4963,8 +5019,10 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="186" t="n">
-        <v>5</v>
+      <c r="B9" s="186" t="inlineStr">
+        <is>
+          <t>T-0005</t>
+        </is>
       </c>
       <c r="C9" s="209" t="n">
         <v>46298</v>
@@ -5017,8 +5075,10 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="187" t="n">
-        <v>6</v>
+      <c r="B10" s="187" t="inlineStr">
+        <is>
+          <t>T-0006</t>
+        </is>
       </c>
       <c r="C10" s="210" t="n">
         <v>46299</v>
@@ -5071,8 +5131,10 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="n">
-        <v>7</v>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>T-0007</t>
+        </is>
       </c>
       <c r="C11" s="209" t="n">
         <v>46299</v>
@@ -5125,8 +5187,10 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="n">
-        <v>8</v>
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>T-0008</t>
+        </is>
       </c>
       <c r="C12" s="210" t="n">
         <v>46299</v>

</xml_diff>

<commit_message>
v6: Торговля test deals (3 Buy, 3 Sell), Дельта formulas
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -2328,32 +2328,28 @@
       </c>
       <c r="E5" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="F5" s="176" t="n">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="G5" s="177" t="n">
-        <v>0.0521</v>
+        <v>62000</v>
       </c>
       <c r="H5" s="178" t="n">
-        <v>0.02605</v>
-      </c>
-      <c r="I5" s="176" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="J5" s="177" t="n">
-        <v>0.0534</v>
-      </c>
-      <c r="K5" s="178" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="L5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="M5" s="177" t="n">
-        <v>2.5</v>
+        <v>6187.6</v>
+      </c>
+      <c r="I5" s="176" t="n"/>
+      <c r="J5" s="177" t="n"/>
+      <c r="K5" s="178" t="n"/>
+      <c r="L5" s="176">
+        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND(MIN(F5,I5)*(K5/I5-H5/F5),8),"")</f>
+        <v/>
+      </c>
+      <c r="M5" s="177">
+        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND((K5/I5)/(H5/F5)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -2363,7 +2359,7 @@
         </is>
       </c>
       <c r="C6" s="210" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="D6" s="187" t="inlineStr">
         <is>
@@ -2372,32 +2368,34 @@
       </c>
       <c r="E6" s="181" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>ETH/USDT</t>
         </is>
       </c>
       <c r="F6" s="182" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="G6" s="183" t="n">
-        <v>62000</v>
+        <v>3200</v>
       </c>
       <c r="H6" s="184" t="n">
-        <v>15500</v>
+        <v>6387.2</v>
       </c>
       <c r="I6" s="182" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="J6" s="183" t="n">
-        <v>64000</v>
+        <v>3350</v>
       </c>
       <c r="K6" s="184" t="n">
-        <v>16000</v>
-      </c>
-      <c r="L6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="M6" s="183" t="n">
-        <v>3.23</v>
+        <v>3343.3</v>
+      </c>
+      <c r="L6" s="182">
+        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND(MIN(F6,I6)*(K6/I6-H6/F6),8),"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="183">
+        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND((K6/I6)/(H6/F6)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -2407,7 +2405,7 @@
         </is>
       </c>
       <c r="C7" s="209" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="D7" s="186" t="inlineStr">
         <is>
@@ -2426,22 +2424,24 @@
         <v>145</v>
       </c>
       <c r="H7" s="178" t="n">
-        <v>2900</v>
+        <v>2894.2</v>
       </c>
       <c r="I7" s="176" t="n">
         <v>20</v>
       </c>
       <c r="J7" s="177" t="n">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="K7" s="178" t="n">
-        <v>2780</v>
-      </c>
-      <c r="L7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="M7" s="177" t="n">
-        <v>-4.14</v>
+        <v>3033.92</v>
+      </c>
+      <c r="L7" s="176">
+        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND(MIN(F7,I7)*(K7/I7-H7/F7),8),"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="177">
+        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND((K7/I7)/(H7/F7)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -2460,32 +2460,28 @@
       </c>
       <c r="E8" s="181" t="inlineStr">
         <is>
-          <t>ETH/USDT</t>
-        </is>
-      </c>
-      <c r="F8" s="182" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G8" s="183" t="n">
-        <v>3200</v>
-      </c>
-      <c r="H8" s="184" t="n">
-        <v>3840</v>
-      </c>
+          <t>ETH/BTC</t>
+        </is>
+      </c>
+      <c r="F8" s="182" t="n"/>
+      <c r="G8" s="183" t="n"/>
+      <c r="H8" s="184" t="n"/>
       <c r="I8" s="182" t="n">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="J8" s="183" t="n">
-        <v>3350</v>
+        <v>0.0525</v>
       </c>
       <c r="K8" s="184" t="n">
-        <v>4020</v>
-      </c>
-      <c r="L8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="M8" s="183" t="n">
-        <v>4.69</v>
+        <v>0.0785925</v>
+      </c>
+      <c r="L8" s="182">
+        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND(MIN(F8,I8)*(K8/I8-H8/F8),8),"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="183">
+        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND((K8/I8)/(H8/F8)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -2495,7 +2491,7 @@
         </is>
       </c>
       <c r="C9" s="209" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D9" s="186" t="inlineStr">
         <is>
@@ -2508,28 +2504,30 @@
         </is>
       </c>
       <c r="F9" s="176" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G9" s="177" t="n">
-        <v>590</v>
+        <v>585</v>
       </c>
       <c r="H9" s="178" t="n">
-        <v>2950</v>
+        <v>1167.66</v>
       </c>
       <c r="I9" s="176" t="n">
         <v>5</v>
       </c>
       <c r="J9" s="177" t="n">
-        <v>575</v>
+        <v>600</v>
       </c>
       <c r="K9" s="178" t="n">
-        <v>2875</v>
-      </c>
-      <c r="L9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="M9" s="177" t="n">
-        <v>-2.54</v>
+        <v>2994</v>
+      </c>
+      <c r="L9" s="176">
+        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND(MIN(F9,I9)*(K9/I9-H9/F9),8),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="177">
+        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND((K9/I9)/(H9/F9)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -2552,116 +2550,70 @@
         </is>
       </c>
       <c r="F10" s="182" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G10" s="183" t="n">
-        <v>62500</v>
+        <v>62200</v>
       </c>
       <c r="H10" s="184" t="n">
-        <v>6250</v>
+        <v>3103.78</v>
       </c>
       <c r="I10" s="182" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J10" s="183" t="n">
-        <v>63100</v>
+        <v>63000</v>
       </c>
       <c r="K10" s="184" t="n">
-        <v>6310</v>
-      </c>
-      <c r="L10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="M10" s="183" t="n">
-        <v>0.96</v>
+        <v>3143.7</v>
+      </c>
+      <c r="L10" s="182">
+        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND(MIN(F10,I10)*(K10/I10-H10/F10),8),"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="183">
+        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND((K10/I10)/(H10/F10)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="inlineStr">
-        <is>
-          <t>T-0007</t>
-        </is>
-      </c>
-      <c r="C11" s="209" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D11" s="186" t="inlineStr">
-        <is>
-          <t>Binance</t>
-        </is>
-      </c>
-      <c r="E11" s="175" t="inlineStr">
-        <is>
-          <t>ETH/BTC</t>
-        </is>
-      </c>
-      <c r="F11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G11" s="177" t="n">
-        <v>0.0518</v>
-      </c>
-      <c r="H11" s="178" t="n">
-        <v>0.04144</v>
-      </c>
-      <c r="I11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="J11" s="177" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="K11" s="178" t="n">
-        <v>0.0424</v>
-      </c>
-      <c r="L11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="M11" s="177" t="n">
-        <v>2.32</v>
+      <c r="B11" s="186" t="n"/>
+      <c r="C11" s="209" t="n"/>
+      <c r="D11" s="186" t="n"/>
+      <c r="E11" s="175" t="n"/>
+      <c r="F11" s="176" t="n"/>
+      <c r="G11" s="177" t="n"/>
+      <c r="H11" s="178" t="n"/>
+      <c r="I11" s="176" t="n"/>
+      <c r="J11" s="177" t="n"/>
+      <c r="K11" s="178" t="n"/>
+      <c r="L11" s="176">
+        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND(MIN(F11,I11)*(K11/I11-H11/F11),8),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="177">
+        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND((K11/I11)/(H11/F11)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="inlineStr">
-        <is>
-          <t>T-0008</t>
-        </is>
-      </c>
-      <c r="C12" s="210" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D12" s="187" t="inlineStr">
-        <is>
-          <t>Bybit</t>
-        </is>
-      </c>
-      <c r="E12" s="181" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="F12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="G12" s="183" t="n">
-        <v>142</v>
-      </c>
-      <c r="H12" s="184" t="n">
-        <v>2130</v>
-      </c>
-      <c r="I12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="J12" s="183" t="n">
-        <v>147</v>
-      </c>
-      <c r="K12" s="184" t="n">
-        <v>2205</v>
-      </c>
-      <c r="L12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="M12" s="183" t="n">
-        <v>3.52</v>
+      <c r="B12" s="187" t="n"/>
+      <c r="C12" s="210" t="n"/>
+      <c r="D12" s="187" t="n"/>
+      <c r="E12" s="181" t="n"/>
+      <c r="F12" s="182" t="n"/>
+      <c r="G12" s="183" t="n"/>
+      <c r="H12" s="184" t="n"/>
+      <c r="I12" s="182" t="n"/>
+      <c r="J12" s="183" t="n"/>
+      <c r="K12" s="184" t="n"/>
+      <c r="L12" s="182">
+        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND(MIN(F12,I12)*(K12/I12-H12/F12),8),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="183">
+        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND((K12/I12)/(H12/F12)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2794,11 +2746,13 @@
       <c r="H5" s="178" t="n">
         <v>0.0267</v>
       </c>
-      <c r="I5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="J5" s="178" t="n">
-        <v>2.5</v>
+      <c r="I5" s="176">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND(MIN(C5,F5)*(H5/F5-E5/C5),8),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="178">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND((H5/F5)/(E5/C5)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K5" s="176" t="n">
         <v>0.00063</v>
@@ -2834,11 +2788,13 @@
       <c r="H6" s="184" t="n">
         <v>16000</v>
       </c>
-      <c r="I6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="J6" s="184" t="n">
-        <v>3.23</v>
+      <c r="I6" s="182">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND(MIN(C6,F6)*(H6/F6-E6/C6),8),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="184">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND((H6/F6)/(E6/C6)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K6" s="182" t="n">
         <v>485</v>
@@ -2874,11 +2830,13 @@
       <c r="H7" s="178" t="n">
         <v>2780</v>
       </c>
-      <c r="I7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="J7" s="178" t="n">
-        <v>-4.14</v>
+      <c r="I7" s="176">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND(MIN(C7,F7)*(H7/F7-E7/C7),8),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="178">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND((H7/F7)/(E7/C7)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K7" s="176" t="n">
         <v>-125</v>
@@ -2914,11 +2872,13 @@
       <c r="H8" s="184" t="n">
         <v>4020</v>
       </c>
-      <c r="I8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="J8" s="184" t="n">
-        <v>4.69</v>
+      <c r="I8" s="182">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND(MIN(C8,F8)*(H8/F8-E8/C8),8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="184">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND((H8/F8)/(E8/C8)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K8" s="182" t="n">
         <v>175</v>
@@ -2954,11 +2914,13 @@
       <c r="H9" s="178" t="n">
         <v>2875</v>
       </c>
-      <c r="I9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="J9" s="178" t="n">
-        <v>-2.54</v>
+      <c r="I9" s="176">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND(MIN(C9,F9)*(H9/F9-E9/C9),8),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="178">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND((H9/F9)/(E9/C9)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K9" s="176" t="n">
         <v>-80</v>
@@ -2994,11 +2956,13 @@
       <c r="H10" s="184" t="n">
         <v>6310</v>
       </c>
-      <c r="I10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="J10" s="184" t="n">
-        <v>0.96</v>
+      <c r="I10" s="182">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND(MIN(C10,F10)*(H10/F10-E10/C10),8),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="184">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND((H10/F10)/(E10/C10)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K10" s="182" t="n">
         <v>55</v>
@@ -3034,11 +2998,13 @@
       <c r="H11" s="178" t="n">
         <v>0.0424</v>
       </c>
-      <c r="I11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="J11" s="178" t="n">
-        <v>2.32</v>
+      <c r="I11" s="176">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND(MIN(C11,F11)*(H11/F11-E11/C11),8),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="178">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND((H11/F11)/(E11/C11)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K11" s="176" t="n">
         <v>0.00092</v>
@@ -3074,11 +3040,13 @@
       <c r="H12" s="184" t="n">
         <v>2205</v>
       </c>
-      <c r="I12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="J12" s="184" t="n">
-        <v>3.52</v>
+      <c r="I12" s="182">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND(MIN(C12,F12)*(H12/F12-E12/C12),8),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="184">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND((H12/F12)/(E12/C12)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K12" s="182" t="n">
         <v>70</v>
@@ -3233,11 +3201,13 @@
       <c r="K5" s="178" t="n">
         <v>0.0267</v>
       </c>
-      <c r="L5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="M5" s="177" t="n">
-        <v>2.5</v>
+      <c r="L5" s="176">
+        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND(MIN(F5,I5)*(K5/I5-H5/F5),8),"")</f>
+        <v/>
+      </c>
+      <c r="M5" s="177">
+        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND((K5/I5)/(H5/F5)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
@@ -3277,11 +3247,13 @@
       <c r="K6" s="184" t="n">
         <v>16000</v>
       </c>
-      <c r="L6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="M6" s="183" t="n">
-        <v>3.23</v>
+      <c r="L6" s="182">
+        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND(MIN(F6,I6)*(K6/I6-H6/F6),8),"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="183">
+        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND((K6/I6)/(H6/F6)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
@@ -3321,11 +3293,13 @@
       <c r="K7" s="178" t="n">
         <v>2780</v>
       </c>
-      <c r="L7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="M7" s="177" t="n">
-        <v>-4.14</v>
+      <c r="L7" s="176">
+        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND(MIN(F7,I7)*(K7/I7-H7/F7),8),"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="177">
+        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND((K7/I7)/(H7/F7)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
@@ -3365,11 +3339,13 @@
       <c r="K8" s="184" t="n">
         <v>4020</v>
       </c>
-      <c r="L8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="M8" s="183" t="n">
-        <v>4.69</v>
+      <c r="L8" s="182">
+        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND(MIN(F8,I8)*(K8/I8-H8/F8),8),"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="183">
+        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND((K8/I8)/(H8/F8)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
@@ -3409,11 +3385,13 @@
       <c r="K9" s="178" t="n">
         <v>2875</v>
       </c>
-      <c r="L9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="M9" s="177" t="n">
-        <v>-2.54</v>
+      <c r="L9" s="176">
+        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND(MIN(F9,I9)*(K9/I9-H9/F9),8),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="177">
+        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND((K9/I9)/(H9/F9)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
@@ -3453,11 +3431,13 @@
       <c r="K10" s="184" t="n">
         <v>6310</v>
       </c>
-      <c r="L10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="M10" s="183" t="n">
-        <v>0.96</v>
+      <c r="L10" s="182">
+        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND(MIN(F10,I10)*(K10/I10-H10/F10),8),"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="183">
+        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND((K10/I10)/(H10/F10)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
@@ -3497,11 +3477,13 @@
       <c r="K11" s="178" t="n">
         <v>0.0424</v>
       </c>
-      <c r="L11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="M11" s="177" t="n">
-        <v>2.32</v>
+      <c r="L11" s="176">
+        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND(MIN(F11,I11)*(K11/I11-H11/F11),8),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="177">
+        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND((K11/I11)/(H11/F11)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -3541,11 +3523,13 @@
       <c r="K12" s="184" t="n">
         <v>2205</v>
       </c>
-      <c r="L12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="M12" s="183" t="n">
-        <v>3.52</v>
+      <c r="L12" s="182">
+        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND(MIN(F12,I12)*(K12/I12-H12/F12),8),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="183">
+        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND((K12/I12)/(H12/F12)*100-100,2),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3678,11 +3662,13 @@
       <c r="H5" s="178" t="n">
         <v>0.0267</v>
       </c>
-      <c r="I5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="J5" s="178" t="n">
-        <v>2.5</v>
+      <c r="I5" s="176">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND(MIN(C5,F5)*(H5/F5-E5/C5),8),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="178">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND((H5/F5)/(E5/C5)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K5" s="176" t="n">
         <v>0.00063</v>
@@ -3718,11 +3704,13 @@
       <c r="H6" s="184" t="n">
         <v>16000</v>
       </c>
-      <c r="I6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="J6" s="184" t="n">
-        <v>3.23</v>
+      <c r="I6" s="182">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND(MIN(C6,F6)*(H6/F6-E6/C6),8),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="184">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND((H6/F6)/(E6/C6)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K6" s="182" t="n">
         <v>485</v>
@@ -3758,11 +3746,13 @@
       <c r="H7" s="178" t="n">
         <v>2780</v>
       </c>
-      <c r="I7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="J7" s="178" t="n">
-        <v>-4.14</v>
+      <c r="I7" s="176">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND(MIN(C7,F7)*(H7/F7-E7/C7),8),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="178">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND((H7/F7)/(E7/C7)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K7" s="176" t="n">
         <v>-125</v>
@@ -3798,11 +3788,13 @@
       <c r="H8" s="184" t="n">
         <v>4020</v>
       </c>
-      <c r="I8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="J8" s="184" t="n">
-        <v>4.69</v>
+      <c r="I8" s="182">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND(MIN(C8,F8)*(H8/F8-E8/C8),8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="184">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND((H8/F8)/(E8/C8)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K8" s="182" t="n">
         <v>175</v>
@@ -3838,11 +3830,13 @@
       <c r="H9" s="178" t="n">
         <v>2875</v>
       </c>
-      <c r="I9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="J9" s="178" t="n">
-        <v>-2.54</v>
+      <c r="I9" s="176">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND(MIN(C9,F9)*(H9/F9-E9/C9),8),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="178">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND((H9/F9)/(E9/C9)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K9" s="176" t="n">
         <v>-80</v>
@@ -3878,11 +3872,13 @@
       <c r="H10" s="184" t="n">
         <v>6310</v>
       </c>
-      <c r="I10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="J10" s="184" t="n">
-        <v>0.96</v>
+      <c r="I10" s="182">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND(MIN(C10,F10)*(H10/F10-E10/C10),8),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="184">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND((H10/F10)/(E10/C10)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K10" s="182" t="n">
         <v>55</v>
@@ -3918,11 +3914,13 @@
       <c r="H11" s="178" t="n">
         <v>0.0424</v>
       </c>
-      <c r="I11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="J11" s="178" t="n">
-        <v>2.32</v>
+      <c r="I11" s="176">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND(MIN(C11,F11)*(H11/F11-E11/C11),8),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="178">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND((H11/F11)/(E11/C11)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K11" s="176" t="n">
         <v>0.00092</v>
@@ -3958,11 +3956,13 @@
       <c r="H12" s="184" t="n">
         <v>2205</v>
       </c>
-      <c r="I12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="J12" s="184" t="n">
-        <v>3.52</v>
+      <c r="I12" s="182">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND(MIN(C12,F12)*(H12/F12-E12/C12),8),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="184">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND((H12/F12)/(E12/C12)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K12" s="182" t="n">
         <v>70</v>
@@ -4834,11 +4834,13 @@
       <c r="L5" s="178" t="n">
         <v>0.0267</v>
       </c>
-      <c r="M5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="N5" s="178" t="n">
-        <v>2.5</v>
+      <c r="M5" s="176">
+        <f>IF(AND(AND(ISNUMBER(G5),ISNUMBER(J5),ISNUMBER(I5),ISNUMBER(L5)),G5&gt;0,J5&gt;0,I5&lt;&gt;0),ROUND(MIN(G5,J5)*(L5/J5-I5/G5),8),"")</f>
+        <v/>
+      </c>
+      <c r="N5" s="178">
+        <f>IF(AND(AND(ISNUMBER(G5),ISNUMBER(J5),ISNUMBER(I5),ISNUMBER(L5)),G5&gt;0,J5&gt;0,I5&lt;&gt;0),ROUND((L5/J5)/(I5/G5)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O5" s="176" t="n">
         <v>0.00063</v>
@@ -4890,11 +4892,13 @@
       <c r="L6" s="184" t="n">
         <v>16000</v>
       </c>
-      <c r="M6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="N6" s="184" t="n">
-        <v>3.23</v>
+      <c r="M6" s="182">
+        <f>IF(AND(AND(ISNUMBER(G6),ISNUMBER(J6),ISNUMBER(I6),ISNUMBER(L6)),G6&gt;0,J6&gt;0,I6&lt;&gt;0),ROUND(MIN(G6,J6)*(L6/J6-I6/G6),8),"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="184">
+        <f>IF(AND(AND(ISNUMBER(G6),ISNUMBER(J6),ISNUMBER(I6),ISNUMBER(L6)),G6&gt;0,J6&gt;0,I6&lt;&gt;0),ROUND((L6/J6)/(I6/G6)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O6" s="182" t="n">
         <v>485</v>
@@ -4946,11 +4950,13 @@
       <c r="L7" s="178" t="n">
         <v>2780</v>
       </c>
-      <c r="M7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="N7" s="178" t="n">
-        <v>-4.14</v>
+      <c r="M7" s="176">
+        <f>IF(AND(AND(ISNUMBER(G7),ISNUMBER(J7),ISNUMBER(I7),ISNUMBER(L7)),G7&gt;0,J7&gt;0,I7&lt;&gt;0),ROUND(MIN(G7,J7)*(L7/J7-I7/G7),8),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="178">
+        <f>IF(AND(AND(ISNUMBER(G7),ISNUMBER(J7),ISNUMBER(I7),ISNUMBER(L7)),G7&gt;0,J7&gt;0,I7&lt;&gt;0),ROUND((L7/J7)/(I7/G7)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O7" s="176" t="n">
         <v>-125</v>
@@ -5002,11 +5008,13 @@
       <c r="L8" s="184" t="n">
         <v>4020</v>
       </c>
-      <c r="M8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="N8" s="184" t="n">
-        <v>4.69</v>
+      <c r="M8" s="182">
+        <f>IF(AND(AND(ISNUMBER(G8),ISNUMBER(J8),ISNUMBER(I8),ISNUMBER(L8)),G8&gt;0,J8&gt;0,I8&lt;&gt;0),ROUND(MIN(G8,J8)*(L8/J8-I8/G8),8),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="184">
+        <f>IF(AND(AND(ISNUMBER(G8),ISNUMBER(J8),ISNUMBER(I8),ISNUMBER(L8)),G8&gt;0,J8&gt;0,I8&lt;&gt;0),ROUND((L8/J8)/(I8/G8)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O8" s="182" t="n">
         <v>175</v>
@@ -5058,11 +5066,13 @@
       <c r="L9" s="178" t="n">
         <v>2875</v>
       </c>
-      <c r="M9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="N9" s="178" t="n">
-        <v>-2.54</v>
+      <c r="M9" s="176">
+        <f>IF(AND(AND(ISNUMBER(G9),ISNUMBER(J9),ISNUMBER(I9),ISNUMBER(L9)),G9&gt;0,J9&gt;0,I9&lt;&gt;0),ROUND(MIN(G9,J9)*(L9/J9-I9/G9),8),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="178">
+        <f>IF(AND(AND(ISNUMBER(G9),ISNUMBER(J9),ISNUMBER(I9),ISNUMBER(L9)),G9&gt;0,J9&gt;0,I9&lt;&gt;0),ROUND((L9/J9)/(I9/G9)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O9" s="176" t="n">
         <v>-80</v>
@@ -5114,11 +5124,13 @@
       <c r="L10" s="184" t="n">
         <v>6310</v>
       </c>
-      <c r="M10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="N10" s="184" t="n">
-        <v>0.96</v>
+      <c r="M10" s="182">
+        <f>IF(AND(AND(ISNUMBER(G10),ISNUMBER(J10),ISNUMBER(I10),ISNUMBER(L10)),G10&gt;0,J10&gt;0,I10&lt;&gt;0),ROUND(MIN(G10,J10)*(L10/J10-I10/G10),8),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="184">
+        <f>IF(AND(AND(ISNUMBER(G10),ISNUMBER(J10),ISNUMBER(I10),ISNUMBER(L10)),G10&gt;0,J10&gt;0,I10&lt;&gt;0),ROUND((L10/J10)/(I10/G10)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O10" s="182" t="n">
         <v>55</v>
@@ -5170,11 +5182,13 @@
       <c r="L11" s="178" t="n">
         <v>0.0424</v>
       </c>
-      <c r="M11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="N11" s="178" t="n">
-        <v>2.32</v>
+      <c r="M11" s="176">
+        <f>IF(AND(AND(ISNUMBER(G11),ISNUMBER(J11),ISNUMBER(I11),ISNUMBER(L11)),G11&gt;0,J11&gt;0,I11&lt;&gt;0),ROUND(MIN(G11,J11)*(L11/J11-I11/G11),8),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="178">
+        <f>IF(AND(AND(ISNUMBER(G11),ISNUMBER(J11),ISNUMBER(I11),ISNUMBER(L11)),G11&gt;0,J11&gt;0,I11&lt;&gt;0),ROUND((L11/J11)/(I11/G11)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O11" s="176" t="n">
         <v>0.00092</v>
@@ -5226,11 +5240,13 @@
       <c r="L12" s="184" t="n">
         <v>2205</v>
       </c>
-      <c r="M12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="N12" s="184" t="n">
-        <v>3.52</v>
+      <c r="M12" s="182">
+        <f>IF(AND(AND(ISNUMBER(G12),ISNUMBER(J12),ISNUMBER(I12),ISNUMBER(L12)),G12&gt;0,J12&gt;0,I12&lt;&gt;0),ROUND(MIN(G12,J12)*(L12/J12-I12/G12),8),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="184">
+        <f>IF(AND(AND(ISNUMBER(G12),ISNUMBER(J12),ISNUMBER(I12),ISNUMBER(L12)),G12&gt;0,J12&gt;0,I12&lt;&gt;0),ROUND((L12/J12)/(I12/G12)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="O12" s="182" t="n">
         <v>70</v>
@@ -5372,11 +5388,13 @@
       <c r="H5" s="178" t="n">
         <v>0.0267</v>
       </c>
-      <c r="I5" s="176" t="n">
-        <v>0.00065</v>
-      </c>
-      <c r="J5" s="178" t="n">
-        <v>2.5</v>
+      <c r="I5" s="176">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND(MIN(C5,F5)*(H5/F5-E5/C5),8),"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="178">
+        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND((H5/F5)/(E5/C5)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K5" s="176" t="n">
         <v>0.00063</v>
@@ -5412,11 +5430,13 @@
       <c r="H6" s="184" t="n">
         <v>16000</v>
       </c>
-      <c r="I6" s="182" t="n">
-        <v>500</v>
-      </c>
-      <c r="J6" s="184" t="n">
-        <v>3.23</v>
+      <c r="I6" s="182">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND(MIN(C6,F6)*(H6/F6-E6/C6),8),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="184">
+        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND((H6/F6)/(E6/C6)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K6" s="182" t="n">
         <v>485</v>
@@ -5452,11 +5472,13 @@
       <c r="H7" s="178" t="n">
         <v>2780</v>
       </c>
-      <c r="I7" s="176" t="n">
-        <v>-120</v>
-      </c>
-      <c r="J7" s="178" t="n">
-        <v>-4.14</v>
+      <c r="I7" s="176">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND(MIN(C7,F7)*(H7/F7-E7/C7),8),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="178">
+        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND((H7/F7)/(E7/C7)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K7" s="176" t="n">
         <v>-125</v>
@@ -5492,11 +5514,13 @@
       <c r="H8" s="184" t="n">
         <v>4020</v>
       </c>
-      <c r="I8" s="182" t="n">
-        <v>180</v>
-      </c>
-      <c r="J8" s="184" t="n">
-        <v>4.69</v>
+      <c r="I8" s="182">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND(MIN(C8,F8)*(H8/F8-E8/C8),8),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="184">
+        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND((H8/F8)/(E8/C8)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K8" s="182" t="n">
         <v>175</v>
@@ -5532,11 +5556,13 @@
       <c r="H9" s="178" t="n">
         <v>2875</v>
       </c>
-      <c r="I9" s="176" t="n">
-        <v>-75</v>
-      </c>
-      <c r="J9" s="178" t="n">
-        <v>-2.54</v>
+      <c r="I9" s="176">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND(MIN(C9,F9)*(H9/F9-E9/C9),8),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="178">
+        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND((H9/F9)/(E9/C9)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K9" s="176" t="n">
         <v>-80</v>
@@ -5572,11 +5598,13 @@
       <c r="H10" s="184" t="n">
         <v>6310</v>
       </c>
-      <c r="I10" s="182" t="n">
-        <v>60</v>
-      </c>
-      <c r="J10" s="184" t="n">
-        <v>0.96</v>
+      <c r="I10" s="182">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND(MIN(C10,F10)*(H10/F10-E10/C10),8),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="184">
+        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND((H10/F10)/(E10/C10)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K10" s="182" t="n">
         <v>55</v>
@@ -5612,11 +5640,13 @@
       <c r="H11" s="178" t="n">
         <v>0.0424</v>
       </c>
-      <c r="I11" s="176" t="n">
-        <v>0.00096</v>
-      </c>
-      <c r="J11" s="178" t="n">
-        <v>2.32</v>
+      <c r="I11" s="176">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND(MIN(C11,F11)*(H11/F11-E11/C11),8),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="178">
+        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND((H11/F11)/(E11/C11)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K11" s="176" t="n">
         <v>0.00092</v>
@@ -5652,11 +5682,13 @@
       <c r="H12" s="184" t="n">
         <v>2205</v>
       </c>
-      <c r="I12" s="182" t="n">
-        <v>75</v>
-      </c>
-      <c r="J12" s="184" t="n">
-        <v>3.52</v>
+      <c r="I12" s="182">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND(MIN(C12,F12)*(H12/F12-E12/C12),8),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="184">
+        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND((H12/F12)/(E12/C12)*100-100,2),"")</f>
+        <v/>
       </c>
       <c r="K12" s="182" t="n">
         <v>70</v>

</xml_diff>

<commit_message>
v6: 12 test deals incl. same-pair groups, sort by Пара, Закрытые and ИТОГО Торговля aligned
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -22,8 +22,8 @@
     <definedName name="Список_Протокол">OFFSET(Справочники!$B$5,0,0,MAX(1,COUNTA(Справочники!$B$5:$B$104)),1)</definedName>
     <definedName name="Список_Действие_Торговля">OFFSET(Справочники!$C$5,0,0,MAX(1,COUNTA(Справочники!$C$5:$C$104)),1)</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Ввод'!$A$1:$K$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Торговля'!$B$4:$M$12</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Торговля'!$A$1:$N$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Торговля'!$B$4:$M$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Торговля'!$A$1:$N$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ИТОГО Торговля'!$B$4:$M$12</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'ИТОГО Торговля'!$A$1:$N$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Лэндинг'!$B$4:$M$12</definedName>
@@ -2223,7 +2223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:M12"/>
+  <dimension ref="B1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -2315,34 +2315,40 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="186" t="inlineStr">
         <is>
-          <t>T-0001</t>
+          <t>T-0005</t>
         </is>
       </c>
       <c r="C5" s="209" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="D5" s="186" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="E5" s="175" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>BNB/USDT</t>
         </is>
       </c>
       <c r="F5" s="176" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="G5" s="177" t="n">
-        <v>62000</v>
+        <v>585</v>
       </c>
       <c r="H5" s="178" t="n">
-        <v>6187.6</v>
-      </c>
-      <c r="I5" s="176" t="n"/>
-      <c r="J5" s="177" t="n"/>
-      <c r="K5" s="178" t="n"/>
+        <v>1167.66</v>
+      </c>
+      <c r="I5" s="176" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" s="177" t="n">
+        <v>600</v>
+      </c>
+      <c r="K5" s="178" t="n">
+        <v>2994</v>
+      </c>
       <c r="L5" s="176">
         <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND(MIN(F5,I5)*(K5/I5-H5/F5),8),"")</f>
         <v/>
@@ -2355,40 +2361,34 @@
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="187" t="inlineStr">
         <is>
-          <t>T-0002</t>
+          <t>T-0001</t>
         </is>
       </c>
       <c r="C6" s="210" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="D6" s="187" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E6" s="181" t="inlineStr">
         <is>
-          <t>ETH/USDT</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="F6" s="182" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="G6" s="183" t="n">
-        <v>3200</v>
+        <v>62000</v>
       </c>
       <c r="H6" s="184" t="n">
-        <v>6387.2</v>
-      </c>
-      <c r="I6" s="182" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="183" t="n">
-        <v>3350</v>
-      </c>
-      <c r="K6" s="184" t="n">
-        <v>3343.3</v>
-      </c>
+        <v>6187.6</v>
+      </c>
+      <c r="I6" s="182" t="n"/>
+      <c r="J6" s="183" t="n"/>
+      <c r="K6" s="184" t="n"/>
       <c r="L6" s="182">
         <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND(MIN(F6,I6)*(K6/I6-H6/F6),8),"")</f>
         <v/>
@@ -2401,11 +2401,11 @@
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="186" t="inlineStr">
         <is>
-          <t>T-0003</t>
+          <t>T-0006</t>
         </is>
       </c>
       <c r="C7" s="209" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D7" s="186" t="inlineStr">
         <is>
@@ -2414,26 +2414,26 @@
       </c>
       <c r="E7" s="175" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="F7" s="176" t="n">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="G7" s="177" t="n">
-        <v>145</v>
+        <v>62200</v>
       </c>
       <c r="H7" s="178" t="n">
-        <v>2894.2</v>
+        <v>3103.78</v>
       </c>
       <c r="I7" s="176" t="n">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="J7" s="177" t="n">
-        <v>152</v>
+        <v>63000</v>
       </c>
       <c r="K7" s="178" t="n">
-        <v>3033.92</v>
+        <v>3143.7</v>
       </c>
       <c r="L7" s="176">
         <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND(MIN(F7,I7)*(K7/I7-H7/F7),8),"")</f>
@@ -2487,11 +2487,11 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="186" t="inlineStr">
         <is>
-          <t>T-0005</t>
+          <t>T-0002</t>
         </is>
       </c>
       <c r="C9" s="209" t="n">
-        <v>46299</v>
+        <v>46297</v>
       </c>
       <c r="D9" s="186" t="inlineStr">
         <is>
@@ -2500,26 +2500,26 @@
       </c>
       <c r="E9" s="175" t="inlineStr">
         <is>
-          <t>BNB/USDT</t>
+          <t>ETH/USDT</t>
         </is>
       </c>
       <c r="F9" s="176" t="n">
         <v>2</v>
       </c>
       <c r="G9" s="177" t="n">
-        <v>585</v>
+        <v>3200</v>
       </c>
       <c r="H9" s="178" t="n">
-        <v>1167.66</v>
+        <v>6387.2</v>
       </c>
       <c r="I9" s="176" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J9" s="177" t="n">
-        <v>600</v>
+        <v>3350</v>
       </c>
       <c r="K9" s="178" t="n">
-        <v>2994</v>
+        <v>3343.3</v>
       </c>
       <c r="L9" s="176">
         <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND(MIN(F9,I9)*(K9/I9-H9/F9),8),"")</f>
@@ -2533,40 +2533,34 @@
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="187" t="inlineStr">
         <is>
-          <t>T-0006</t>
+          <t>T-0007</t>
         </is>
       </c>
       <c r="C10" s="210" t="n">
-        <v>46299</v>
+        <v>46300</v>
       </c>
       <c r="D10" s="187" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E10" s="181" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>ETH/USDT</t>
         </is>
       </c>
       <c r="F10" s="182" t="n">
-        <v>0.05</v>
+        <v>1.2</v>
       </c>
       <c r="G10" s="183" t="n">
-        <v>62200</v>
+        <v>3180</v>
       </c>
       <c r="H10" s="184" t="n">
-        <v>3103.78</v>
-      </c>
-      <c r="I10" s="182" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="J10" s="183" t="n">
-        <v>63000</v>
-      </c>
-      <c r="K10" s="184" t="n">
-        <v>3143.7</v>
-      </c>
+        <v>3808.368</v>
+      </c>
+      <c r="I10" s="182" t="n"/>
+      <c r="J10" s="183" t="n"/>
+      <c r="K10" s="184" t="n"/>
       <c r="L10" s="182">
         <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND(MIN(F10,I10)*(K10/I10-H10/F10),8),"")</f>
         <v/>
@@ -2577,13 +2571,33 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="n"/>
-      <c r="C11" s="209" t="n"/>
-      <c r="D11" s="186" t="n"/>
-      <c r="E11" s="175" t="n"/>
-      <c r="F11" s="176" t="n"/>
-      <c r="G11" s="177" t="n"/>
-      <c r="H11" s="178" t="n"/>
+      <c r="B11" s="186" t="inlineStr">
+        <is>
+          <t>T-0008</t>
+        </is>
+      </c>
+      <c r="C11" s="209" t="n">
+        <v>46300</v>
+      </c>
+      <c r="D11" s="186" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="E11" s="175" t="inlineStr">
+        <is>
+          <t>ETH/USDT</t>
+        </is>
+      </c>
+      <c r="F11" s="176" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G11" s="177" t="n">
+        <v>3250</v>
+      </c>
+      <c r="H11" s="178" t="n">
+        <v>2594.8</v>
+      </c>
       <c r="I11" s="176" t="n"/>
       <c r="J11" s="177" t="n"/>
       <c r="K11" s="178" t="n"/>
@@ -2597,16 +2611,36 @@
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="n"/>
-      <c r="C12" s="210" t="n"/>
-      <c r="D12" s="187" t="n"/>
-      <c r="E12" s="181" t="n"/>
+      <c r="B12" s="187" t="inlineStr">
+        <is>
+          <t>T-0009</t>
+        </is>
+      </c>
+      <c r="C12" s="210" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D12" s="187" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="E12" s="181" t="inlineStr">
+        <is>
+          <t>ETH/USDT</t>
+        </is>
+      </c>
       <c r="F12" s="182" t="n"/>
       <c r="G12" s="183" t="n"/>
       <c r="H12" s="184" t="n"/>
-      <c r="I12" s="182" t="n"/>
-      <c r="J12" s="183" t="n"/>
-      <c r="K12" s="184" t="n"/>
+      <c r="I12" s="182" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J12" s="183" t="n">
+        <v>3400</v>
+      </c>
+      <c r="K12" s="184" t="n">
+        <v>5089.8</v>
+      </c>
       <c r="L12" s="182">
         <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND(MIN(F12,I12)*(K12/I12-H12/F12),8),"")</f>
         <v/>
@@ -2616,8 +2650,178 @@
         <v/>
       </c>
     </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="B13" s="186" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
+      </c>
+      <c r="C13" s="209" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D13" s="186" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="E13" s="175" t="inlineStr">
+        <is>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="F13" s="176" t="n">
+        <v>20</v>
+      </c>
+      <c r="G13" s="177" t="n">
+        <v>145</v>
+      </c>
+      <c r="H13" s="178" t="n">
+        <v>2894.2</v>
+      </c>
+      <c r="I13" s="176" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" s="177" t="n">
+        <v>152</v>
+      </c>
+      <c r="K13" s="178" t="n">
+        <v>3033.92</v>
+      </c>
+      <c r="L13" s="176">
+        <f>IF(AND(AND(ISNUMBER(F13),ISNUMBER(I13),ISNUMBER(H13),ISNUMBER(K13)),F13&gt;0,I13&gt;0,H13&lt;&gt;0),ROUND(MIN(F13,I13)*(K13/I13-H13/F13),8),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="177">
+        <f>IF(AND(AND(ISNUMBER(F13),ISNUMBER(I13),ISNUMBER(H13),ISNUMBER(K13)),F13&gt;0,I13&gt;0,H13&lt;&gt;0),ROUND((K13/I13)/(H13/F13)*100-100,2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="B14" s="187" t="inlineStr">
+        <is>
+          <t>T-0010</t>
+        </is>
+      </c>
+      <c r="C14" s="210" t="n">
+        <v>46300</v>
+      </c>
+      <c r="D14" s="187" t="inlineStr">
+        <is>
+          <t>Binance</t>
+        </is>
+      </c>
+      <c r="E14" s="181" t="inlineStr">
+        <is>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="F14" s="182" t="n"/>
+      <c r="G14" s="183" t="n"/>
+      <c r="H14" s="184" t="n"/>
+      <c r="I14" s="182" t="n">
+        <v>30</v>
+      </c>
+      <c r="J14" s="183" t="n">
+        <v>150</v>
+      </c>
+      <c r="K14" s="184" t="n">
+        <v>4491</v>
+      </c>
+      <c r="L14" s="182">
+        <f>IF(AND(AND(ISNUMBER(F14),ISNUMBER(I14),ISNUMBER(H14),ISNUMBER(K14)),F14&gt;0,I14&gt;0,H14&lt;&gt;0),ROUND(MIN(F14,I14)*(K14/I14-H14/F14),8),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="183">
+        <f>IF(AND(AND(ISNUMBER(F14),ISNUMBER(I14),ISNUMBER(H14),ISNUMBER(K14)),F14&gt;0,I14&gt;0,H14&lt;&gt;0),ROUND((K14/I14)/(H14/F14)*100-100,2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="B15" s="186" t="inlineStr">
+        <is>
+          <t>T-0011</t>
+        </is>
+      </c>
+      <c r="C15" s="209" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D15" s="186" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="E15" s="175" t="inlineStr">
+        <is>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="F15" s="176" t="n"/>
+      <c r="G15" s="177" t="n"/>
+      <c r="H15" s="178" t="n"/>
+      <c r="I15" s="176" t="n">
+        <v>10</v>
+      </c>
+      <c r="J15" s="177" t="n">
+        <v>152</v>
+      </c>
+      <c r="K15" s="178" t="n">
+        <v>1516.96</v>
+      </c>
+      <c r="L15" s="176">
+        <f>IF(AND(AND(ISNUMBER(F15),ISNUMBER(I15),ISNUMBER(H15),ISNUMBER(K15)),F15&gt;0,I15&gt;0,H15&lt;&gt;0),ROUND(MIN(F15,I15)*(K15/I15-H15/F15),8),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="177">
+        <f>IF(AND(AND(ISNUMBER(F15),ISNUMBER(I15),ISNUMBER(H15),ISNUMBER(K15)),F15&gt;0,I15&gt;0,H15&lt;&gt;0),ROUND((K15/I15)/(H15/F15)*100-100,2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="B16" s="187" t="inlineStr">
+        <is>
+          <t>T-0012</t>
+        </is>
+      </c>
+      <c r="C16" s="210" t="n">
+        <v>46301</v>
+      </c>
+      <c r="D16" s="187" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="E16" s="181" t="inlineStr">
+        <is>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="F16" s="182" t="n">
+        <v>25</v>
+      </c>
+      <c r="G16" s="183" t="n">
+        <v>146</v>
+      </c>
+      <c r="H16" s="184" t="n">
+        <v>3642.7</v>
+      </c>
+      <c r="I16" s="182" t="n"/>
+      <c r="J16" s="183" t="n"/>
+      <c r="K16" s="184" t="n"/>
+      <c r="L16" s="182">
+        <f>IF(AND(AND(ISNUMBER(F16),ISNUMBER(I16),ISNUMBER(H16),ISNUMBER(K16)),F16&gt;0,I16&gt;0,H16&lt;&gt;0),ROUND(MIN(F16,I16)*(K16/I16-H16/F16),8),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="183">
+        <f>IF(AND(AND(ISNUMBER(F16),ISNUMBER(I16),ISNUMBER(H16),ISNUMBER(K16)),F16&gt;0,I16&gt;0,H16&lt;&gt;0),ROUND((K16/I16)/(H16/F16)*100-100,2),"")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B4:M12"/>
+  <autoFilter ref="B4:M16">
+    <sortState ref="B5:M16">
+      <sortCondition ref="E5:E16"/>
+    </sortState>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>
@@ -2725,26 +2929,32 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
-        </is>
-      </c>
-      <c r="C5" s="176" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="177" t="n">
-        <v>0.0521</v>
-      </c>
-      <c r="E5" s="178" t="n">
-        <v>0.02605</v>
-      </c>
-      <c r="F5" s="176" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G5" s="177" t="n">
-        <v>0.0534</v>
-      </c>
-      <c r="H5" s="178" t="n">
-        <v>0.0267</v>
+          <t>BNB/USDT</t>
+        </is>
+      </c>
+      <c r="C5" s="176">
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5))</f>
+        <v/>
+      </c>
+      <c r="D5" s="177">
+        <f>IF(C5="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C5)</f>
+        <v/>
+      </c>
+      <c r="E5" s="178">
+        <f>IF(C5="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B5))</f>
+        <v/>
+      </c>
+      <c r="F5" s="176">
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5))</f>
+        <v/>
+      </c>
+      <c r="G5" s="177">
+        <f>IF(F5="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="178">
+        <f>IF(F5="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B5))</f>
+        <v/>
       </c>
       <c r="I5" s="176">
         <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND(MIN(C5,F5)*(H5/F5-E5/C5),8),"")</f>
@@ -2754,15 +2964,9 @@
         <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND((H5/F5)/(E5/C5)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K5" s="176" t="n">
-        <v>0.00063</v>
-      </c>
-      <c r="L5" s="177" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="M5" s="177" t="n">
-        <v>0.0522</v>
-      </c>
+      <c r="K5" s="176" t="n"/>
+      <c r="L5" s="177" t="n"/>
+      <c r="M5" s="177" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="181" t="inlineStr">
@@ -2770,23 +2974,29 @@
           <t>BTC/USDT</t>
         </is>
       </c>
-      <c r="C6" s="182" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D6" s="183" t="n">
-        <v>62000</v>
-      </c>
-      <c r="E6" s="184" t="n">
-        <v>15500</v>
-      </c>
-      <c r="F6" s="182" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="G6" s="183" t="n">
-        <v>64000</v>
-      </c>
-      <c r="H6" s="184" t="n">
-        <v>16000</v>
+      <c r="C6" s="182">
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6))</f>
+        <v/>
+      </c>
+      <c r="D6" s="183">
+        <f>IF(C6="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C6)</f>
+        <v/>
+      </c>
+      <c r="E6" s="184">
+        <f>IF(C6="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B6))</f>
+        <v/>
+      </c>
+      <c r="F6" s="182">
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6))</f>
+        <v/>
+      </c>
+      <c r="G6" s="183">
+        <f>IF(F6="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="184">
+        <f>IF(F6="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B6))</f>
+        <v/>
       </c>
       <c r="I6" s="182">
         <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND(MIN(C6,F6)*(H6/F6-E6/C6),8),"")</f>
@@ -2796,39 +3006,39 @@
         <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND((H6/F6)/(E6/C6)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K6" s="182" t="n">
-        <v>485</v>
-      </c>
-      <c r="L6" s="183" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="M6" s="183" t="n">
-        <v>62155</v>
-      </c>
+      <c r="K6" s="182" t="n"/>
+      <c r="L6" s="183" t="n"/>
+      <c r="M6" s="183" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="175" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="C7" s="176" t="n">
-        <v>20</v>
-      </c>
-      <c r="D7" s="177" t="n">
-        <v>145</v>
-      </c>
-      <c r="E7" s="178" t="n">
-        <v>2900</v>
-      </c>
-      <c r="F7" s="176" t="n">
-        <v>20</v>
-      </c>
-      <c r="G7" s="177" t="n">
-        <v>139</v>
-      </c>
-      <c r="H7" s="178" t="n">
-        <v>2780</v>
+          <t>ETH/BTC</t>
+        </is>
+      </c>
+      <c r="C7" s="176">
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7))</f>
+        <v/>
+      </c>
+      <c r="D7" s="177">
+        <f>IF(C7="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C7)</f>
+        <v/>
+      </c>
+      <c r="E7" s="178">
+        <f>IF(C7="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B7))</f>
+        <v/>
+      </c>
+      <c r="F7" s="176">
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7))</f>
+        <v/>
+      </c>
+      <c r="G7" s="177">
+        <f>IF(F7="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="178">
+        <f>IF(F7="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B7))</f>
+        <v/>
       </c>
       <c r="I7" s="176">
         <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND(MIN(C7,F7)*(H7/F7-E7/C7),8),"")</f>
@@ -2838,15 +3048,9 @@
         <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND((H7/F7)/(E7/C7)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K7" s="176" t="n">
-        <v>-125</v>
-      </c>
-      <c r="L7" s="177" t="n">
-        <v>-4.31</v>
-      </c>
-      <c r="M7" s="177" t="n">
-        <v>145.3</v>
-      </c>
+      <c r="K7" s="176" t="n"/>
+      <c r="L7" s="177" t="n"/>
+      <c r="M7" s="177" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="181" t="inlineStr">
@@ -2854,23 +3058,29 @@
           <t>ETH/USDT</t>
         </is>
       </c>
-      <c r="C8" s="182" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="D8" s="183" t="n">
-        <v>3200</v>
-      </c>
-      <c r="E8" s="184" t="n">
-        <v>3840</v>
-      </c>
-      <c r="F8" s="182" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="G8" s="183" t="n">
-        <v>3350</v>
-      </c>
-      <c r="H8" s="184" t="n">
-        <v>4020</v>
+      <c r="C8" s="182">
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8))</f>
+        <v/>
+      </c>
+      <c r="D8" s="183">
+        <f>IF(C8="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="184">
+        <f>IF(C8="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B8))</f>
+        <v/>
+      </c>
+      <c r="F8" s="182">
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8))</f>
+        <v/>
+      </c>
+      <c r="G8" s="183">
+        <f>IF(F8="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="184">
+        <f>IF(F8="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B8))</f>
+        <v/>
       </c>
       <c r="I8" s="182">
         <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND(MIN(C8,F8)*(H8/F8-E8/C8),8),"")</f>
@@ -2880,39 +3090,39 @@
         <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND((H8/F8)/(E8/C8)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K8" s="182" t="n">
-        <v>175</v>
-      </c>
-      <c r="L8" s="183" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="M8" s="183" t="n">
-        <v>3203.84</v>
-      </c>
+      <c r="K8" s="182" t="n"/>
+      <c r="L8" s="183" t="n"/>
+      <c r="M8" s="183" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="175" t="inlineStr">
         <is>
-          <t>BNB/USDT</t>
-        </is>
-      </c>
-      <c r="C9" s="176" t="n">
-        <v>5</v>
-      </c>
-      <c r="D9" s="177" t="n">
-        <v>590</v>
-      </c>
-      <c r="E9" s="178" t="n">
-        <v>2950</v>
-      </c>
-      <c r="F9" s="176" t="n">
-        <v>5</v>
-      </c>
-      <c r="G9" s="177" t="n">
-        <v>575</v>
-      </c>
-      <c r="H9" s="178" t="n">
-        <v>2875</v>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="C9" s="176">
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9))</f>
+        <v/>
+      </c>
+      <c r="D9" s="177">
+        <f>IF(C9="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C9)</f>
+        <v/>
+      </c>
+      <c r="E9" s="178">
+        <f>IF(C9="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B9))</f>
+        <v/>
+      </c>
+      <c r="F9" s="176">
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9))</f>
+        <v/>
+      </c>
+      <c r="G9" s="177">
+        <f>IF(F9="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="178">
+        <f>IF(F9="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B9))</f>
+        <v/>
       </c>
       <c r="I9" s="176">
         <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND(MIN(C9,F9)*(H9/F9-E9/C9),8),"")</f>
@@ -2922,40 +3132,18 @@
         <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND((H9/F9)/(E9/C9)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K9" s="176" t="n">
-        <v>-80</v>
-      </c>
-      <c r="L9" s="177" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="M9" s="177" t="n">
-        <v>590.6</v>
-      </c>
+      <c r="K9" s="176" t="n"/>
+      <c r="L9" s="177" t="n"/>
+      <c r="M9" s="177" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="181" t="inlineStr">
-        <is>
-          <t>BTC/USDT</t>
-        </is>
-      </c>
-      <c r="C10" s="182" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D10" s="183" t="n">
-        <v>62500</v>
-      </c>
-      <c r="E10" s="184" t="n">
-        <v>6250</v>
-      </c>
-      <c r="F10" s="182" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G10" s="183" t="n">
-        <v>63100</v>
-      </c>
-      <c r="H10" s="184" t="n">
-        <v>6310</v>
-      </c>
+      <c r="B10" s="181" t="n"/>
+      <c r="C10" s="182" t="n"/>
+      <c r="D10" s="183" t="n"/>
+      <c r="E10" s="184" t="n"/>
+      <c r="F10" s="182" t="n"/>
+      <c r="G10" s="183" t="n"/>
+      <c r="H10" s="184" t="n"/>
       <c r="I10" s="182">
         <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND(MIN(C10,F10)*(H10/F10-E10/C10),8),"")</f>
         <v/>
@@ -2964,40 +3152,18 @@
         <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND((H10/F10)/(E10/C10)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K10" s="182" t="n">
-        <v>55</v>
-      </c>
-      <c r="L10" s="183" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="M10" s="183" t="n">
-        <v>62512.5</v>
-      </c>
+      <c r="K10" s="182" t="n"/>
+      <c r="L10" s="183" t="n"/>
+      <c r="M10" s="183" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="175" t="inlineStr">
-        <is>
-          <t>ETH/BTC</t>
-        </is>
-      </c>
-      <c r="C11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="D11" s="177" t="n">
-        <v>0.0518</v>
-      </c>
-      <c r="E11" s="178" t="n">
-        <v>0.04144</v>
-      </c>
-      <c r="F11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G11" s="177" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="H11" s="178" t="n">
-        <v>0.0424</v>
-      </c>
+      <c r="B11" s="175" t="n"/>
+      <c r="C11" s="176" t="n"/>
+      <c r="D11" s="177" t="n"/>
+      <c r="E11" s="178" t="n"/>
+      <c r="F11" s="176" t="n"/>
+      <c r="G11" s="177" t="n"/>
+      <c r="H11" s="178" t="n"/>
       <c r="I11" s="176">
         <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND(MIN(C11,F11)*(H11/F11-E11/C11),8),"")</f>
         <v/>
@@ -3006,40 +3172,18 @@
         <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND((H11/F11)/(E11/C11)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K11" s="176" t="n">
-        <v>0.00092</v>
-      </c>
-      <c r="L11" s="177" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="M11" s="177" t="n">
-        <v>0.05185</v>
-      </c>
+      <c r="K11" s="176" t="n"/>
+      <c r="L11" s="177" t="n"/>
+      <c r="M11" s="177" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="181" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="C12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="D12" s="183" t="n">
-        <v>142</v>
-      </c>
-      <c r="E12" s="184" t="n">
-        <v>2130</v>
-      </c>
-      <c r="F12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="G12" s="183" t="n">
-        <v>147</v>
-      </c>
-      <c r="H12" s="184" t="n">
-        <v>2205</v>
-      </c>
+      <c r="B12" s="181" t="n"/>
+      <c r="C12" s="182" t="n"/>
+      <c r="D12" s="183" t="n"/>
+      <c r="E12" s="184" t="n"/>
+      <c r="F12" s="182" t="n"/>
+      <c r="G12" s="183" t="n"/>
+      <c r="H12" s="184" t="n"/>
       <c r="I12" s="182">
         <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND(MIN(C12,F12)*(H12/F12-E12/C12),8),"")</f>
         <v/>
@@ -3048,15 +3192,9 @@
         <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND((H12/F12)/(E12/C12)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="K12" s="182" t="n">
-        <v>70</v>
-      </c>
-      <c r="L12" s="183" t="n">
-        <v>3.29</v>
-      </c>
-      <c r="M12" s="183" t="n">
-        <v>142.28</v>
-      </c>
+      <c r="K12" s="182" t="n"/>
+      <c r="L12" s="183" t="n"/>
+      <c r="M12" s="183" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:M12"/>
@@ -3167,39 +3305,39 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="186" t="inlineStr">
         <is>
-          <t>L-0001</t>
+          <t>L-0005</t>
         </is>
       </c>
       <c r="C5" s="209" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="D5" s="186" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="E5" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>BNB/USDT</t>
         </is>
       </c>
       <c r="F5" s="176" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G5" s="177" t="n">
-        <v>0.0521</v>
+        <v>590</v>
       </c>
       <c r="H5" s="178" t="n">
-        <v>0.02605</v>
+        <v>2950</v>
       </c>
       <c r="I5" s="176" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="J5" s="177" t="n">
-        <v>0.0534</v>
+        <v>575</v>
       </c>
       <c r="K5" s="178" t="n">
-        <v>0.0267</v>
+        <v>2875</v>
       </c>
       <c r="L5" s="176">
         <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND(MIN(F5,I5)*(K5/I5-H5/F5),8),"")</f>
@@ -3259,11 +3397,11 @@
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="186" t="inlineStr">
         <is>
-          <t>L-0003</t>
+          <t>L-0006</t>
         </is>
       </c>
       <c r="C7" s="209" t="n">
-        <v>46297</v>
+        <v>46299</v>
       </c>
       <c r="D7" s="186" t="inlineStr">
         <is>
@@ -3272,26 +3410,26 @@
       </c>
       <c r="E7" s="175" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="F7" s="176" t="n">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="G7" s="177" t="n">
-        <v>145</v>
+        <v>62500</v>
       </c>
       <c r="H7" s="178" t="n">
-        <v>2900</v>
+        <v>6250</v>
       </c>
       <c r="I7" s="176" t="n">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="J7" s="177" t="n">
-        <v>139</v>
+        <v>63100</v>
       </c>
       <c r="K7" s="178" t="n">
-        <v>2780</v>
+        <v>6310</v>
       </c>
       <c r="L7" s="176">
         <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND(MIN(F7,I7)*(K7/I7-H7/F7),8),"")</f>
@@ -3305,11 +3443,11 @@
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="187" t="inlineStr">
         <is>
-          <t>L-0004</t>
+          <t>L-0001</t>
         </is>
       </c>
       <c r="C8" s="210" t="n">
-        <v>46298</v>
+        <v>46296</v>
       </c>
       <c r="D8" s="187" t="inlineStr">
         <is>
@@ -3318,26 +3456,26 @@
       </c>
       <c r="E8" s="181" t="inlineStr">
         <is>
-          <t>ETH/USDT</t>
+          <t>ETH/BTC</t>
         </is>
       </c>
       <c r="F8" s="182" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="G8" s="183" t="n">
-        <v>3200</v>
+        <v>0.0521</v>
       </c>
       <c r="H8" s="184" t="n">
-        <v>3840</v>
+        <v>0.02605</v>
       </c>
       <c r="I8" s="182" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
       <c r="J8" s="183" t="n">
-        <v>3350</v>
+        <v>0.0534</v>
       </c>
       <c r="K8" s="184" t="n">
-        <v>4020</v>
+        <v>0.0267</v>
       </c>
       <c r="L8" s="182">
         <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND(MIN(F8,I8)*(K8/I8-H8/F8),8),"")</f>
@@ -3351,39 +3489,39 @@
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="186" t="inlineStr">
         <is>
-          <t>L-0005</t>
+          <t>L-0007</t>
         </is>
       </c>
       <c r="C9" s="209" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D9" s="186" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E9" s="175" t="inlineStr">
         <is>
-          <t>BNB/USDT</t>
+          <t>ETH/BTC</t>
         </is>
       </c>
       <c r="F9" s="176" t="n">
-        <v>5</v>
+        <v>0.8</v>
       </c>
       <c r="G9" s="177" t="n">
-        <v>590</v>
+        <v>0.0518</v>
       </c>
       <c r="H9" s="178" t="n">
-        <v>2950</v>
+        <v>0.04144</v>
       </c>
       <c r="I9" s="176" t="n">
-        <v>5</v>
+        <v>0.8</v>
       </c>
       <c r="J9" s="177" t="n">
-        <v>575</v>
+        <v>0.053</v>
       </c>
       <c r="K9" s="178" t="n">
-        <v>2875</v>
+        <v>0.0424</v>
       </c>
       <c r="L9" s="176">
         <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND(MIN(F9,I9)*(K9/I9-H9/F9),8),"")</f>
@@ -3397,39 +3535,39 @@
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="187" t="inlineStr">
         <is>
-          <t>L-0006</t>
+          <t>L-0004</t>
         </is>
       </c>
       <c r="C10" s="210" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="D10" s="187" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E10" s="181" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>ETH/USDT</t>
         </is>
       </c>
       <c r="F10" s="182" t="n">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="G10" s="183" t="n">
-        <v>62500</v>
+        <v>3200</v>
       </c>
       <c r="H10" s="184" t="n">
-        <v>6250</v>
+        <v>3840</v>
       </c>
       <c r="I10" s="182" t="n">
-        <v>0.1</v>
+        <v>1.2</v>
       </c>
       <c r="J10" s="183" t="n">
-        <v>63100</v>
+        <v>3350</v>
       </c>
       <c r="K10" s="184" t="n">
-        <v>6310</v>
+        <v>4020</v>
       </c>
       <c r="L10" s="182">
         <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND(MIN(F10,I10)*(K10/I10-H10/F10),8),"")</f>
@@ -3443,39 +3581,39 @@
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="186" t="inlineStr">
         <is>
-          <t>L-0007</t>
+          <t>L-0003</t>
         </is>
       </c>
       <c r="C11" s="209" t="n">
-        <v>46299</v>
+        <v>46297</v>
       </c>
       <c r="D11" s="186" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>OKX</t>
         </is>
       </c>
       <c r="E11" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>SOL/USDT</t>
         </is>
       </c>
       <c r="F11" s="176" t="n">
-        <v>0.8</v>
+        <v>20</v>
       </c>
       <c r="G11" s="177" t="n">
-        <v>0.0518</v>
+        <v>145</v>
       </c>
       <c r="H11" s="178" t="n">
-        <v>0.04144</v>
+        <v>2900</v>
       </c>
       <c r="I11" s="176" t="n">
-        <v>0.8</v>
+        <v>20</v>
       </c>
       <c r="J11" s="177" t="n">
-        <v>0.053</v>
+        <v>139</v>
       </c>
       <c r="K11" s="178" t="n">
-        <v>0.0424</v>
+        <v>2780</v>
       </c>
       <c r="L11" s="176">
         <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND(MIN(F11,I11)*(K11/I11-H11/F11),8),"")</f>
@@ -3533,7 +3671,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:M12"/>
+  <autoFilter ref="B4:M12">
+    <sortState ref="B5:M12">
+      <sortCondition ref="E5:E12"/>
+    </sortState>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>
@@ -4047,111 +4189,111 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="186" t="inlineStr">
         <is>
-          <t>P-0001</t>
+          <t>P-0003</t>
         </is>
       </c>
       <c r="C5" s="209" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="D5" s="186" t="inlineStr">
         <is>
-          <t>Uniswap</t>
+          <t>PancakeSwap</t>
         </is>
       </c>
       <c r="E5" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>BNB/USDT</t>
         </is>
       </c>
       <c r="F5" s="176" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G5" s="177" t="n">
-        <v>0.104</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="187" t="inlineStr">
         <is>
-          <t>P-0002</t>
+          <t>P-0006</t>
         </is>
       </c>
       <c r="C6" s="210" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="D6" s="187" t="inlineStr">
         <is>
-          <t>Raydium</t>
+          <t>Uniswap</t>
         </is>
       </c>
       <c r="E6" s="181" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="F6" s="182" t="n">
-        <v>30</v>
+        <v>0.05</v>
       </c>
       <c r="G6" s="183" t="n">
-        <v>4350</v>
+        <v>3125</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="186" t="inlineStr">
         <is>
-          <t>P-0003</t>
+          <t>P-0001</t>
         </is>
       </c>
       <c r="C7" s="209" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="D7" s="186" t="inlineStr">
         <is>
-          <t>PancakeSwap</t>
+          <t>Uniswap</t>
         </is>
       </c>
       <c r="E7" s="175" t="inlineStr">
         <is>
-          <t>BNB/USDT</t>
+          <t>ETH/BTC</t>
         </is>
       </c>
       <c r="F7" s="176" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G7" s="177" t="n">
-        <v>2360</v>
+        <v>0.104</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="187" t="inlineStr">
         <is>
-          <t>P-0004</t>
+          <t>P-0007</t>
         </is>
       </c>
       <c r="C8" s="210" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D8" s="187" t="inlineStr">
         <is>
-          <t>Uniswap</t>
+          <t>PancakeSwap</t>
         </is>
       </c>
       <c r="E8" s="181" t="inlineStr">
         <is>
-          <t>ETH/USDT</t>
+          <t>ETH/BTC</t>
         </is>
       </c>
       <c r="F8" s="182" t="n">
-        <v>1.5</v>
+        <v>1.2</v>
       </c>
       <c r="G8" s="183" t="n">
-        <v>4800</v>
+        <v>0.0624</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="186" t="inlineStr">
         <is>
-          <t>P-0005</t>
+          <t>P-0004</t>
         </is>
       </c>
       <c r="C9" s="209" t="n">
@@ -4159,71 +4301,71 @@
       </c>
       <c r="D9" s="186" t="inlineStr">
         <is>
-          <t>Orca</t>
+          <t>Uniswap</t>
         </is>
       </c>
       <c r="E9" s="175" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
+          <t>ETH/USDT</t>
         </is>
       </c>
       <c r="F9" s="176" t="n">
-        <v>12</v>
+        <v>1.5</v>
       </c>
       <c r="G9" s="177" t="n">
-        <v>1740</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="187" t="inlineStr">
         <is>
-          <t>P-0006</t>
+          <t>P-0002</t>
         </is>
       </c>
       <c r="C10" s="210" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="D10" s="187" t="inlineStr">
         <is>
-          <t>Uniswap</t>
+          <t>Raydium</t>
         </is>
       </c>
       <c r="E10" s="181" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>SOL/USDT</t>
         </is>
       </c>
       <c r="F10" s="182" t="n">
-        <v>0.05</v>
+        <v>30</v>
       </c>
       <c r="G10" s="183" t="n">
-        <v>3125</v>
+        <v>4350</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="186" t="inlineStr">
         <is>
-          <t>P-0007</t>
+          <t>P-0005</t>
         </is>
       </c>
       <c r="C11" s="209" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="D11" s="186" t="inlineStr">
         <is>
-          <t>PancakeSwap</t>
+          <t>Orca</t>
         </is>
       </c>
       <c r="E11" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>SOL/USDT</t>
         </is>
       </c>
       <c r="F11" s="176" t="n">
-        <v>1.2</v>
+        <v>12</v>
       </c>
       <c r="G11" s="177" t="n">
-        <v>0.0624</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
@@ -4253,7 +4395,11 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:G12"/>
+  <autoFilter ref="B4:G12">
+    <sortState ref="B5:G12">
+      <sortCondition ref="E5:E12"/>
+    </sortState>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:G2"/>
   </mergeCells>
@@ -4797,42 +4943,42 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="186" t="inlineStr">
         <is>
-          <t>T-0001</t>
+          <t>T-0006</t>
         </is>
       </c>
       <c r="C5" s="209" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="D5" s="209" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="E5" s="186" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>OKX</t>
         </is>
       </c>
       <c r="F5" s="175" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="G5" s="176" t="n">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="H5" s="177" t="n">
-        <v>0.0521</v>
+        <v>62200</v>
       </c>
       <c r="I5" s="178" t="n">
-        <v>0.02605</v>
+        <v>3103.78</v>
       </c>
       <c r="J5" s="176" t="n">
-        <v>0.5</v>
+        <v>0.05</v>
       </c>
       <c r="K5" s="177" t="n">
-        <v>0.0534</v>
+        <v>63000</v>
       </c>
       <c r="L5" s="178" t="n">
-        <v>0.0267</v>
+        <v>3143.7</v>
       </c>
       <c r="M5" s="176">
         <f>IF(AND(AND(ISNUMBER(G5),ISNUMBER(J5),ISNUMBER(I5),ISNUMBER(L5)),G5&gt;0,J5&gt;0,I5&lt;&gt;0),ROUND(MIN(G5,J5)*(L5/J5-I5/G5),8),"")</f>
@@ -4842,55 +4988,49 @@
         <f>IF(AND(AND(ISNUMBER(G5),ISNUMBER(J5),ISNUMBER(I5),ISNUMBER(L5)),G5&gt;0,J5&gt;0,I5&lt;&gt;0),ROUND((L5/J5)/(I5/G5)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O5" s="176" t="n">
-        <v>0.00063</v>
-      </c>
-      <c r="P5" s="177" t="n">
-        <v>2.42</v>
-      </c>
-      <c r="Q5" s="177" t="n">
-        <v>0.0522</v>
-      </c>
+      <c r="O5" s="176" t="n"/>
+      <c r="P5" s="177" t="n"/>
+      <c r="Q5" s="177" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="187" t="inlineStr">
         <is>
-          <t>T-0002</t>
+          <t>T-0003</t>
         </is>
       </c>
       <c r="C6" s="210" t="n">
-        <v>46296</v>
+        <v>46298</v>
       </c>
       <c r="D6" s="210" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="E6" s="187" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>OKX</t>
         </is>
       </c>
       <c r="F6" s="181" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>SOL/USDT</t>
         </is>
       </c>
       <c r="G6" s="182" t="n">
-        <v>0.25</v>
+        <v>20</v>
       </c>
       <c r="H6" s="183" t="n">
-        <v>62000</v>
+        <v>145</v>
       </c>
       <c r="I6" s="184" t="n">
-        <v>15500</v>
+        <v>2894.2</v>
       </c>
       <c r="J6" s="182" t="n">
-        <v>0.25</v>
+        <v>20</v>
       </c>
       <c r="K6" s="183" t="n">
-        <v>64000</v>
+        <v>152</v>
       </c>
       <c r="L6" s="184" t="n">
-        <v>16000</v>
+        <v>3033.92</v>
       </c>
       <c r="M6" s="182">
         <f>IF(AND(AND(ISNUMBER(G6),ISNUMBER(J6),ISNUMBER(I6),ISNUMBER(L6)),G6&gt;0,J6&gt;0,I6&lt;&gt;0),ROUND(MIN(G6,J6)*(L6/J6-I6/G6),8),"")</f>
@@ -4900,56 +5040,22 @@
         <f>IF(AND(AND(ISNUMBER(G6),ISNUMBER(J6),ISNUMBER(I6),ISNUMBER(L6)),G6&gt;0,J6&gt;0,I6&lt;&gt;0),ROUND((L6/J6)/(I6/G6)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O6" s="182" t="n">
-        <v>485</v>
-      </c>
-      <c r="P6" s="183" t="n">
-        <v>3.13</v>
-      </c>
-      <c r="Q6" s="183" t="n">
-        <v>62155</v>
-      </c>
+      <c r="O6" s="182" t="n"/>
+      <c r="P6" s="183" t="n"/>
+      <c r="Q6" s="183" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="inlineStr">
-        <is>
-          <t>T-0003</t>
-        </is>
-      </c>
-      <c r="C7" s="209" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D7" s="209" t="n">
-        <v>46298</v>
-      </c>
-      <c r="E7" s="186" t="inlineStr">
-        <is>
-          <t>OKX</t>
-        </is>
-      </c>
-      <c r="F7" s="175" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="G7" s="176" t="n">
-        <v>20</v>
-      </c>
-      <c r="H7" s="177" t="n">
-        <v>145</v>
-      </c>
-      <c r="I7" s="178" t="n">
-        <v>2900</v>
-      </c>
-      <c r="J7" s="176" t="n">
-        <v>20</v>
-      </c>
-      <c r="K7" s="177" t="n">
-        <v>139</v>
-      </c>
-      <c r="L7" s="178" t="n">
-        <v>2780</v>
-      </c>
+      <c r="B7" s="186" t="n"/>
+      <c r="C7" s="209" t="n"/>
+      <c r="D7" s="209" t="n"/>
+      <c r="E7" s="186" t="n"/>
+      <c r="F7" s="175" t="n"/>
+      <c r="G7" s="176" t="n"/>
+      <c r="H7" s="177" t="n"/>
+      <c r="I7" s="178" t="n"/>
+      <c r="J7" s="176" t="n"/>
+      <c r="K7" s="177" t="n"/>
+      <c r="L7" s="178" t="n"/>
       <c r="M7" s="176">
         <f>IF(AND(AND(ISNUMBER(G7),ISNUMBER(J7),ISNUMBER(I7),ISNUMBER(L7)),G7&gt;0,J7&gt;0,I7&lt;&gt;0),ROUND(MIN(G7,J7)*(L7/J7-I7/G7),8),"")</f>
         <v/>
@@ -4958,56 +5064,22 @@
         <f>IF(AND(AND(ISNUMBER(G7),ISNUMBER(J7),ISNUMBER(I7),ISNUMBER(L7)),G7&gt;0,J7&gt;0,I7&lt;&gt;0),ROUND((L7/J7)/(I7/G7)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O7" s="176" t="n">
-        <v>-125</v>
-      </c>
-      <c r="P7" s="177" t="n">
-        <v>-4.31</v>
-      </c>
-      <c r="Q7" s="177" t="n">
-        <v>145.3</v>
-      </c>
+      <c r="O7" s="176" t="n"/>
+      <c r="P7" s="177" t="n"/>
+      <c r="Q7" s="177" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="inlineStr">
-        <is>
-          <t>T-0004</t>
-        </is>
-      </c>
-      <c r="C8" s="210" t="n">
-        <v>46298</v>
-      </c>
-      <c r="D8" s="210" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E8" s="187" t="inlineStr">
-        <is>
-          <t>Binance</t>
-        </is>
-      </c>
-      <c r="F8" s="181" t="inlineStr">
-        <is>
-          <t>ETH/USDT</t>
-        </is>
-      </c>
-      <c r="G8" s="182" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="H8" s="183" t="n">
-        <v>3200</v>
-      </c>
-      <c r="I8" s="184" t="n">
-        <v>3840</v>
-      </c>
-      <c r="J8" s="182" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="K8" s="183" t="n">
-        <v>3350</v>
-      </c>
-      <c r="L8" s="184" t="n">
-        <v>4020</v>
-      </c>
+      <c r="B8" s="187" t="n"/>
+      <c r="C8" s="210" t="n"/>
+      <c r="D8" s="210" t="n"/>
+      <c r="E8" s="187" t="n"/>
+      <c r="F8" s="181" t="n"/>
+      <c r="G8" s="182" t="n"/>
+      <c r="H8" s="183" t="n"/>
+      <c r="I8" s="184" t="n"/>
+      <c r="J8" s="182" t="n"/>
+      <c r="K8" s="183" t="n"/>
+      <c r="L8" s="184" t="n"/>
       <c r="M8" s="182">
         <f>IF(AND(AND(ISNUMBER(G8),ISNUMBER(J8),ISNUMBER(I8),ISNUMBER(L8)),G8&gt;0,J8&gt;0,I8&lt;&gt;0),ROUND(MIN(G8,J8)*(L8/J8-I8/G8),8),"")</f>
         <v/>
@@ -5016,56 +5088,22 @@
         <f>IF(AND(AND(ISNUMBER(G8),ISNUMBER(J8),ISNUMBER(I8),ISNUMBER(L8)),G8&gt;0,J8&gt;0,I8&lt;&gt;0),ROUND((L8/J8)/(I8/G8)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O8" s="182" t="n">
-        <v>175</v>
-      </c>
-      <c r="P8" s="183" t="n">
-        <v>4.56</v>
-      </c>
-      <c r="Q8" s="183" t="n">
-        <v>3203.84</v>
-      </c>
+      <c r="O8" s="182" t="n"/>
+      <c r="P8" s="183" t="n"/>
+      <c r="Q8" s="183" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="186" t="inlineStr">
-        <is>
-          <t>T-0005</t>
-        </is>
-      </c>
-      <c r="C9" s="209" t="n">
-        <v>46298</v>
-      </c>
-      <c r="D9" s="209" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E9" s="186" t="inlineStr">
-        <is>
-          <t>Bybit</t>
-        </is>
-      </c>
-      <c r="F9" s="175" t="inlineStr">
-        <is>
-          <t>BNB/USDT</t>
-        </is>
-      </c>
-      <c r="G9" s="176" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" s="177" t="n">
-        <v>590</v>
-      </c>
-      <c r="I9" s="178" t="n">
-        <v>2950</v>
-      </c>
-      <c r="J9" s="176" t="n">
-        <v>5</v>
-      </c>
-      <c r="K9" s="177" t="n">
-        <v>575</v>
-      </c>
-      <c r="L9" s="178" t="n">
-        <v>2875</v>
-      </c>
+      <c r="B9" s="186" t="n"/>
+      <c r="C9" s="209" t="n"/>
+      <c r="D9" s="209" t="n"/>
+      <c r="E9" s="186" t="n"/>
+      <c r="F9" s="175" t="n"/>
+      <c r="G9" s="176" t="n"/>
+      <c r="H9" s="177" t="n"/>
+      <c r="I9" s="178" t="n"/>
+      <c r="J9" s="176" t="n"/>
+      <c r="K9" s="177" t="n"/>
+      <c r="L9" s="178" t="n"/>
       <c r="M9" s="176">
         <f>IF(AND(AND(ISNUMBER(G9),ISNUMBER(J9),ISNUMBER(I9),ISNUMBER(L9)),G9&gt;0,J9&gt;0,I9&lt;&gt;0),ROUND(MIN(G9,J9)*(L9/J9-I9/G9),8),"")</f>
         <v/>
@@ -5074,56 +5112,22 @@
         <f>IF(AND(AND(ISNUMBER(G9),ISNUMBER(J9),ISNUMBER(I9),ISNUMBER(L9)),G9&gt;0,J9&gt;0,I9&lt;&gt;0),ROUND((L9/J9)/(I9/G9)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O9" s="176" t="n">
-        <v>-80</v>
-      </c>
-      <c r="P9" s="177" t="n">
-        <v>-2.71</v>
-      </c>
-      <c r="Q9" s="177" t="n">
-        <v>590.6</v>
-      </c>
+      <c r="O9" s="176" t="n"/>
+      <c r="P9" s="177" t="n"/>
+      <c r="Q9" s="177" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="187" t="inlineStr">
-        <is>
-          <t>T-0006</t>
-        </is>
-      </c>
-      <c r="C10" s="210" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D10" s="210" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E10" s="187" t="inlineStr">
-        <is>
-          <t>OKX</t>
-        </is>
-      </c>
-      <c r="F10" s="181" t="inlineStr">
-        <is>
-          <t>BTC/USDT</t>
-        </is>
-      </c>
-      <c r="G10" s="182" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H10" s="183" t="n">
-        <v>62500</v>
-      </c>
-      <c r="I10" s="184" t="n">
-        <v>6250</v>
-      </c>
-      <c r="J10" s="182" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K10" s="183" t="n">
-        <v>63100</v>
-      </c>
-      <c r="L10" s="184" t="n">
-        <v>6310</v>
-      </c>
+      <c r="B10" s="187" t="n"/>
+      <c r="C10" s="210" t="n"/>
+      <c r="D10" s="210" t="n"/>
+      <c r="E10" s="187" t="n"/>
+      <c r="F10" s="181" t="n"/>
+      <c r="G10" s="182" t="n"/>
+      <c r="H10" s="183" t="n"/>
+      <c r="I10" s="184" t="n"/>
+      <c r="J10" s="182" t="n"/>
+      <c r="K10" s="183" t="n"/>
+      <c r="L10" s="184" t="n"/>
       <c r="M10" s="182">
         <f>IF(AND(AND(ISNUMBER(G10),ISNUMBER(J10),ISNUMBER(I10),ISNUMBER(L10)),G10&gt;0,J10&gt;0,I10&lt;&gt;0),ROUND(MIN(G10,J10)*(L10/J10-I10/G10),8),"")</f>
         <v/>
@@ -5132,56 +5136,22 @@
         <f>IF(AND(AND(ISNUMBER(G10),ISNUMBER(J10),ISNUMBER(I10),ISNUMBER(L10)),G10&gt;0,J10&gt;0,I10&lt;&gt;0),ROUND((L10/J10)/(I10/G10)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O10" s="182" t="n">
-        <v>55</v>
-      </c>
-      <c r="P10" s="183" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="Q10" s="183" t="n">
-        <v>62512.5</v>
-      </c>
+      <c r="O10" s="182" t="n"/>
+      <c r="P10" s="183" t="n"/>
+      <c r="Q10" s="183" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="186" t="inlineStr">
-        <is>
-          <t>T-0007</t>
-        </is>
-      </c>
-      <c r="C11" s="209" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D11" s="209" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E11" s="186" t="inlineStr">
-        <is>
-          <t>Binance</t>
-        </is>
-      </c>
-      <c r="F11" s="175" t="inlineStr">
-        <is>
-          <t>ETH/BTC</t>
-        </is>
-      </c>
-      <c r="G11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H11" s="177" t="n">
-        <v>0.0518</v>
-      </c>
-      <c r="I11" s="178" t="n">
-        <v>0.04144</v>
-      </c>
-      <c r="J11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="K11" s="177" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="L11" s="178" t="n">
-        <v>0.0424</v>
-      </c>
+      <c r="B11" s="186" t="n"/>
+      <c r="C11" s="209" t="n"/>
+      <c r="D11" s="209" t="n"/>
+      <c r="E11" s="186" t="n"/>
+      <c r="F11" s="175" t="n"/>
+      <c r="G11" s="176" t="n"/>
+      <c r="H11" s="177" t="n"/>
+      <c r="I11" s="178" t="n"/>
+      <c r="J11" s="176" t="n"/>
+      <c r="K11" s="177" t="n"/>
+      <c r="L11" s="178" t="n"/>
       <c r="M11" s="176">
         <f>IF(AND(AND(ISNUMBER(G11),ISNUMBER(J11),ISNUMBER(I11),ISNUMBER(L11)),G11&gt;0,J11&gt;0,I11&lt;&gt;0),ROUND(MIN(G11,J11)*(L11/J11-I11/G11),8),"")</f>
         <v/>
@@ -5190,56 +5160,22 @@
         <f>IF(AND(AND(ISNUMBER(G11),ISNUMBER(J11),ISNUMBER(I11),ISNUMBER(L11)),G11&gt;0,J11&gt;0,I11&lt;&gt;0),ROUND((L11/J11)/(I11/G11)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O11" s="176" t="n">
-        <v>0.00092</v>
-      </c>
-      <c r="P11" s="177" t="n">
-        <v>2.22</v>
-      </c>
-      <c r="Q11" s="177" t="n">
-        <v>0.05185</v>
-      </c>
+      <c r="O11" s="176" t="n"/>
+      <c r="P11" s="177" t="n"/>
+      <c r="Q11" s="177" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
-      <c r="B12" s="187" t="inlineStr">
-        <is>
-          <t>T-0008</t>
-        </is>
-      </c>
-      <c r="C12" s="210" t="n">
-        <v>46299</v>
-      </c>
-      <c r="D12" s="210" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E12" s="187" t="inlineStr">
-        <is>
-          <t>Bybit</t>
-        </is>
-      </c>
-      <c r="F12" s="181" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="G12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="H12" s="183" t="n">
-        <v>142</v>
-      </c>
-      <c r="I12" s="184" t="n">
-        <v>2130</v>
-      </c>
-      <c r="J12" s="182" t="n">
-        <v>15</v>
-      </c>
-      <c r="K12" s="183" t="n">
-        <v>147</v>
-      </c>
-      <c r="L12" s="184" t="n">
-        <v>2205</v>
-      </c>
+      <c r="B12" s="187" t="n"/>
+      <c r="C12" s="210" t="n"/>
+      <c r="D12" s="210" t="n"/>
+      <c r="E12" s="187" t="n"/>
+      <c r="F12" s="181" t="n"/>
+      <c r="G12" s="182" t="n"/>
+      <c r="H12" s="183" t="n"/>
+      <c r="I12" s="184" t="n"/>
+      <c r="J12" s="182" t="n"/>
+      <c r="K12" s="183" t="n"/>
+      <c r="L12" s="184" t="n"/>
       <c r="M12" s="182">
         <f>IF(AND(AND(ISNUMBER(G12),ISNUMBER(J12),ISNUMBER(I12),ISNUMBER(L12)),G12&gt;0,J12&gt;0,I12&lt;&gt;0),ROUND(MIN(G12,J12)*(L12/J12-I12/G12),8),"")</f>
         <v/>
@@ -5248,15 +5184,9 @@
         <f>IF(AND(AND(ISNUMBER(G12),ISNUMBER(J12),ISNUMBER(I12),ISNUMBER(L12)),G12&gt;0,J12&gt;0,I12&lt;&gt;0),ROUND((L12/J12)/(I12/G12)*100-100,2),"")</f>
         <v/>
       </c>
-      <c r="O12" s="182" t="n">
-        <v>70</v>
-      </c>
-      <c r="P12" s="183" t="n">
-        <v>3.29</v>
-      </c>
-      <c r="Q12" s="183" t="n">
-        <v>142.28</v>
-      </c>
+      <c r="O12" s="182" t="n"/>
+      <c r="P12" s="183" t="n"/>
+      <c r="Q12" s="183" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:Q12"/>

</xml_diff>

<commit_message>
v6: open/closed split (remainder in Торговля, closed part in Закрытые), highlight partial deals, ИТОГО without double count
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -1215,6 +1215,16 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FDE9D9"/>
+          <bgColor rgb="00FDE9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -2331,32 +2341,20 @@
           <t>BNB/USDT</t>
         </is>
       </c>
-      <c r="F5" s="176" t="n">
-        <v>2</v>
-      </c>
-      <c r="G5" s="177" t="n">
-        <v>585</v>
-      </c>
-      <c r="H5" s="178" t="n">
-        <v>1167.66</v>
-      </c>
+      <c r="F5" s="176" t="n"/>
+      <c r="G5" s="177" t="n"/>
+      <c r="H5" s="178" t="n"/>
       <c r="I5" s="176" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="177" t="n">
         <v>600</v>
       </c>
       <c r="K5" s="178" t="n">
-        <v>2994</v>
-      </c>
-      <c r="L5" s="176">
-        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND(MIN(F5,I5)*(K5/I5-H5/F5),8),"")</f>
-        <v/>
-      </c>
-      <c r="M5" s="177">
-        <f>IF(AND(AND(ISNUMBER(F5),ISNUMBER(I5),ISNUMBER(H5),ISNUMBER(K5)),F5&gt;0,I5&gt;0,H5&lt;&gt;0),ROUND((K5/I5)/(H5/F5)*100-100,2),"")</f>
-        <v/>
-      </c>
+        <v>1796.4</v>
+      </c>
+      <c r="L5" s="176" t="n"/>
+      <c r="M5" s="177" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="187" t="inlineStr">
@@ -2389,113 +2387,89 @@
       <c r="I6" s="182" t="n"/>
       <c r="J6" s="183" t="n"/>
       <c r="K6" s="184" t="n"/>
-      <c r="L6" s="182">
-        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND(MIN(F6,I6)*(K6/I6-H6/F6),8),"")</f>
-        <v/>
-      </c>
-      <c r="M6" s="183">
-        <f>IF(AND(AND(ISNUMBER(F6),ISNUMBER(I6),ISNUMBER(H6),ISNUMBER(K6)),F6&gt;0,I6&gt;0,H6&lt;&gt;0),ROUND((K6/I6)/(H6/F6)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="L6" s="182" t="n"/>
+      <c r="M6" s="183" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="B7" s="186" t="inlineStr">
         <is>
-          <t>T-0006</t>
+          <t>T-0004</t>
         </is>
       </c>
       <c r="C7" s="209" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="D7" s="186" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E7" s="175" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
-        </is>
-      </c>
-      <c r="F7" s="176" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G7" s="177" t="n">
-        <v>62200</v>
-      </c>
-      <c r="H7" s="178" t="n">
-        <v>3103.78</v>
-      </c>
+          <t>ETH/BTC</t>
+        </is>
+      </c>
+      <c r="F7" s="176" t="n"/>
+      <c r="G7" s="177" t="n"/>
+      <c r="H7" s="178" t="n"/>
       <c r="I7" s="176" t="n">
-        <v>0.05</v>
+        <v>1.5</v>
       </c>
       <c r="J7" s="177" t="n">
-        <v>63000</v>
+        <v>0.0525</v>
       </c>
       <c r="K7" s="178" t="n">
-        <v>3143.7</v>
-      </c>
-      <c r="L7" s="176">
-        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND(MIN(F7,I7)*(K7/I7-H7/F7),8),"")</f>
-        <v/>
-      </c>
-      <c r="M7" s="177">
-        <f>IF(AND(AND(ISNUMBER(F7),ISNUMBER(I7),ISNUMBER(H7),ISNUMBER(K7)),F7&gt;0,I7&gt;0,H7&lt;&gt;0),ROUND((K7/I7)/(H7/F7)*100-100,2),"")</f>
-        <v/>
-      </c>
+        <v>0.0785925</v>
+      </c>
+      <c r="L7" s="176" t="n"/>
+      <c r="M7" s="177" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="187" t="inlineStr">
         <is>
-          <t>T-0004</t>
+          <t>T-0002</t>
         </is>
       </c>
       <c r="C8" s="210" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="D8" s="187" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="E8" s="181" t="inlineStr">
         <is>
-          <t>ETH/BTC</t>
-        </is>
-      </c>
-      <c r="F8" s="182" t="n"/>
-      <c r="G8" s="183" t="n"/>
-      <c r="H8" s="184" t="n"/>
-      <c r="I8" s="182" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="J8" s="183" t="n">
-        <v>0.0525</v>
-      </c>
-      <c r="K8" s="184" t="n">
-        <v>0.0785925</v>
-      </c>
-      <c r="L8" s="182">
-        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND(MIN(F8,I8)*(K8/I8-H8/F8),8),"")</f>
-        <v/>
-      </c>
-      <c r="M8" s="183">
-        <f>IF(AND(AND(ISNUMBER(F8),ISNUMBER(I8),ISNUMBER(H8),ISNUMBER(K8)),F8&gt;0,I8&gt;0,H8&lt;&gt;0),ROUND((K8/I8)/(H8/F8)*100-100,2),"")</f>
-        <v/>
-      </c>
+          <t>ETH/USDT</t>
+        </is>
+      </c>
+      <c r="F8" s="182" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="183" t="n">
+        <v>3200</v>
+      </c>
+      <c r="H8" s="184" t="n">
+        <v>3193.6</v>
+      </c>
+      <c r="I8" s="182" t="n"/>
+      <c r="J8" s="183" t="n"/>
+      <c r="K8" s="184" t="n"/>
+      <c r="L8" s="182" t="n"/>
+      <c r="M8" s="183" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="B9" s="186" t="inlineStr">
         <is>
-          <t>T-0002</t>
+          <t>T-0007</t>
         </is>
       </c>
       <c r="C9" s="209" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="D9" s="186" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E9" s="175" t="inlineStr">
@@ -2504,36 +2478,24 @@
         </is>
       </c>
       <c r="F9" s="176" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G9" s="177" t="n">
-        <v>3200</v>
+        <v>3180</v>
       </c>
       <c r="H9" s="178" t="n">
-        <v>6387.2</v>
-      </c>
-      <c r="I9" s="176" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="177" t="n">
-        <v>3350</v>
-      </c>
-      <c r="K9" s="178" t="n">
-        <v>3343.3</v>
-      </c>
-      <c r="L9" s="176">
-        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND(MIN(F9,I9)*(K9/I9-H9/F9),8),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="177">
-        <f>IF(AND(AND(ISNUMBER(F9),ISNUMBER(I9),ISNUMBER(H9),ISNUMBER(K9)),F9&gt;0,I9&gt;0,H9&lt;&gt;0),ROUND((K9/I9)/(H9/F9)*100-100,2),"")</f>
-        <v/>
-      </c>
+        <v>3808.368</v>
+      </c>
+      <c r="I9" s="176" t="n"/>
+      <c r="J9" s="177" t="n"/>
+      <c r="K9" s="178" t="n"/>
+      <c r="L9" s="176" t="n"/>
+      <c r="M9" s="177" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="187" t="inlineStr">
         <is>
-          <t>T-0007</t>
+          <t>T-0008</t>
         </is>
       </c>
       <c r="C10" s="210" t="n">
@@ -2541,7 +2503,7 @@
       </c>
       <c r="D10" s="187" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="E10" s="181" t="inlineStr">
@@ -2550,38 +2512,32 @@
         </is>
       </c>
       <c r="F10" s="182" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="G10" s="183" t="n">
-        <v>3180</v>
+        <v>3250</v>
       </c>
       <c r="H10" s="184" t="n">
-        <v>3808.368</v>
+        <v>2594.8</v>
       </c>
       <c r="I10" s="182" t="n"/>
       <c r="J10" s="183" t="n"/>
       <c r="K10" s="184" t="n"/>
-      <c r="L10" s="182">
-        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND(MIN(F10,I10)*(K10/I10-H10/F10),8),"")</f>
-        <v/>
-      </c>
-      <c r="M10" s="183">
-        <f>IF(AND(AND(ISNUMBER(F10),ISNUMBER(I10),ISNUMBER(H10),ISNUMBER(K10)),F10&gt;0,I10&gt;0,H10&lt;&gt;0),ROUND((K10/I10)/(H10/F10)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="L10" s="182" t="n"/>
+      <c r="M10" s="183" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="B11" s="186" t="inlineStr">
         <is>
-          <t>T-0008</t>
+          <t>T-0009</t>
         </is>
       </c>
       <c r="C11" s="209" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="D11" s="186" t="inlineStr">
         <is>
-          <t>Bybit</t>
+          <t>OKX</t>
         </is>
       </c>
       <c r="E11" s="175" t="inlineStr">
@@ -2589,79 +2545,67 @@
           <t>ETH/USDT</t>
         </is>
       </c>
-      <c r="F11" s="176" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G11" s="177" t="n">
-        <v>3250</v>
-      </c>
-      <c r="H11" s="178" t="n">
-        <v>2594.8</v>
-      </c>
-      <c r="I11" s="176" t="n"/>
-      <c r="J11" s="177" t="n"/>
-      <c r="K11" s="178" t="n"/>
-      <c r="L11" s="176">
-        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND(MIN(F11,I11)*(K11/I11-H11/F11),8),"")</f>
-        <v/>
-      </c>
-      <c r="M11" s="177">
-        <f>IF(AND(AND(ISNUMBER(F11),ISNUMBER(I11),ISNUMBER(H11),ISNUMBER(K11)),F11&gt;0,I11&gt;0,H11&lt;&gt;0),ROUND((K11/I11)/(H11/F11)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="F11" s="176" t="n"/>
+      <c r="G11" s="177" t="n"/>
+      <c r="H11" s="178" t="n"/>
+      <c r="I11" s="176" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="J11" s="177" t="n">
+        <v>3400</v>
+      </c>
+      <c r="K11" s="178" t="n">
+        <v>5089.8</v>
+      </c>
+      <c r="L11" s="176" t="n"/>
+      <c r="M11" s="177" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="B12" s="187" t="inlineStr">
         <is>
-          <t>T-0009</t>
+          <t>T-0010</t>
         </is>
       </c>
       <c r="C12" s="210" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="D12" s="187" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Binance</t>
         </is>
       </c>
       <c r="E12" s="181" t="inlineStr">
         <is>
-          <t>ETH/USDT</t>
+          <t>SOL/USDT</t>
         </is>
       </c>
       <c r="F12" s="182" t="n"/>
       <c r="G12" s="183" t="n"/>
       <c r="H12" s="184" t="n"/>
       <c r="I12" s="182" t="n">
-        <v>1.5</v>
+        <v>30</v>
       </c>
       <c r="J12" s="183" t="n">
-        <v>3400</v>
+        <v>150</v>
       </c>
       <c r="K12" s="184" t="n">
-        <v>5089.8</v>
-      </c>
-      <c r="L12" s="182">
-        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND(MIN(F12,I12)*(K12/I12-H12/F12),8),"")</f>
-        <v/>
-      </c>
-      <c r="M12" s="183">
-        <f>IF(AND(AND(ISNUMBER(F12),ISNUMBER(I12),ISNUMBER(H12),ISNUMBER(K12)),F12&gt;0,I12&gt;0,H12&lt;&gt;0),ROUND((K12/I12)/(H12/F12)*100-100,2),"")</f>
-        <v/>
-      </c>
+        <v>4491</v>
+      </c>
+      <c r="L12" s="182" t="n"/>
+      <c r="M12" s="183" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="B13" s="186" t="inlineStr">
         <is>
-          <t>T-0003</t>
+          <t>T-0011</t>
         </is>
       </c>
       <c r="C13" s="209" t="n">
-        <v>46298</v>
+        <v>46301</v>
       </c>
       <c r="D13" s="186" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="E13" s="175" t="inlineStr">
@@ -2669,45 +2613,33 @@
           <t>SOL/USDT</t>
         </is>
       </c>
-      <c r="F13" s="176" t="n">
-        <v>20</v>
-      </c>
-      <c r="G13" s="177" t="n">
-        <v>145</v>
-      </c>
-      <c r="H13" s="178" t="n">
-        <v>2894.2</v>
-      </c>
+      <c r="F13" s="176" t="n"/>
+      <c r="G13" s="177" t="n"/>
+      <c r="H13" s="178" t="n"/>
       <c r="I13" s="176" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J13" s="177" t="n">
         <v>152</v>
       </c>
       <c r="K13" s="178" t="n">
-        <v>3033.92</v>
-      </c>
-      <c r="L13" s="176">
-        <f>IF(AND(AND(ISNUMBER(F13),ISNUMBER(I13),ISNUMBER(H13),ISNUMBER(K13)),F13&gt;0,I13&gt;0,H13&lt;&gt;0),ROUND(MIN(F13,I13)*(K13/I13-H13/F13),8),"")</f>
-        <v/>
-      </c>
-      <c r="M13" s="177">
-        <f>IF(AND(AND(ISNUMBER(F13),ISNUMBER(I13),ISNUMBER(H13),ISNUMBER(K13)),F13&gt;0,I13&gt;0,H13&lt;&gt;0),ROUND((K13/I13)/(H13/F13)*100-100,2),"")</f>
-        <v/>
-      </c>
+        <v>1516.96</v>
+      </c>
+      <c r="L13" s="176" t="n"/>
+      <c r="M13" s="177" t="n"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="B14" s="187" t="inlineStr">
         <is>
-          <t>T-0010</t>
+          <t>T-0012</t>
         </is>
       </c>
       <c r="C14" s="210" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="D14" s="187" t="inlineStr">
         <is>
-          <t>Binance</t>
+          <t>OKX</t>
         </is>
       </c>
       <c r="E14" s="181" t="inlineStr">
@@ -2715,106 +2647,48 @@
           <t>SOL/USDT</t>
         </is>
       </c>
-      <c r="F14" s="182" t="n"/>
-      <c r="G14" s="183" t="n"/>
-      <c r="H14" s="184" t="n"/>
-      <c r="I14" s="182" t="n">
-        <v>30</v>
-      </c>
-      <c r="J14" s="183" t="n">
-        <v>150</v>
-      </c>
-      <c r="K14" s="184" t="n">
-        <v>4491</v>
-      </c>
-      <c r="L14" s="182">
-        <f>IF(AND(AND(ISNUMBER(F14),ISNUMBER(I14),ISNUMBER(H14),ISNUMBER(K14)),F14&gt;0,I14&gt;0,H14&lt;&gt;0),ROUND(MIN(F14,I14)*(K14/I14-H14/F14),8),"")</f>
-        <v/>
-      </c>
-      <c r="M14" s="183">
-        <f>IF(AND(AND(ISNUMBER(F14),ISNUMBER(I14),ISNUMBER(H14),ISNUMBER(K14)),F14&gt;0,I14&gt;0,H14&lt;&gt;0),ROUND((K14/I14)/(H14/F14)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="F14" s="182" t="n">
+        <v>25</v>
+      </c>
+      <c r="G14" s="183" t="n">
+        <v>146</v>
+      </c>
+      <c r="H14" s="184" t="n">
+        <v>3642.7</v>
+      </c>
+      <c r="I14" s="182" t="n"/>
+      <c r="J14" s="183" t="n"/>
+      <c r="K14" s="184" t="n"/>
+      <c r="L14" s="182" t="n"/>
+      <c r="M14" s="183" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="B15" s="186" t="inlineStr">
-        <is>
-          <t>T-0011</t>
-        </is>
-      </c>
-      <c r="C15" s="209" t="n">
-        <v>46301</v>
-      </c>
-      <c r="D15" s="186" t="inlineStr">
-        <is>
-          <t>Bybit</t>
-        </is>
-      </c>
-      <c r="E15" s="175" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
+      <c r="B15" s="186" t="n"/>
+      <c r="C15" s="209" t="n"/>
+      <c r="D15" s="186" t="n"/>
+      <c r="E15" s="175" t="n"/>
       <c r="F15" s="176" t="n"/>
       <c r="G15" s="177" t="n"/>
       <c r="H15" s="178" t="n"/>
-      <c r="I15" s="176" t="n">
-        <v>10</v>
-      </c>
-      <c r="J15" s="177" t="n">
-        <v>152</v>
-      </c>
-      <c r="K15" s="178" t="n">
-        <v>1516.96</v>
-      </c>
-      <c r="L15" s="176">
-        <f>IF(AND(AND(ISNUMBER(F15),ISNUMBER(I15),ISNUMBER(H15),ISNUMBER(K15)),F15&gt;0,I15&gt;0,H15&lt;&gt;0),ROUND(MIN(F15,I15)*(K15/I15-H15/F15),8),"")</f>
-        <v/>
-      </c>
-      <c r="M15" s="177">
-        <f>IF(AND(AND(ISNUMBER(F15),ISNUMBER(I15),ISNUMBER(H15),ISNUMBER(K15)),F15&gt;0,I15&gt;0,H15&lt;&gt;0),ROUND((K15/I15)/(H15/F15)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="I15" s="176" t="n"/>
+      <c r="J15" s="177" t="n"/>
+      <c r="K15" s="178" t="n"/>
+      <c r="L15" s="176" t="n"/>
+      <c r="M15" s="177" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="187" t="inlineStr">
-        <is>
-          <t>T-0012</t>
-        </is>
-      </c>
-      <c r="C16" s="210" t="n">
-        <v>46301</v>
-      </c>
-      <c r="D16" s="187" t="inlineStr">
-        <is>
-          <t>OKX</t>
-        </is>
-      </c>
-      <c r="E16" s="181" t="inlineStr">
-        <is>
-          <t>SOL/USDT</t>
-        </is>
-      </c>
-      <c r="F16" s="182" t="n">
-        <v>25</v>
-      </c>
-      <c r="G16" s="183" t="n">
-        <v>146</v>
-      </c>
-      <c r="H16" s="184" t="n">
-        <v>3642.7</v>
-      </c>
+      <c r="B16" s="187" t="n"/>
+      <c r="C16" s="210" t="n"/>
+      <c r="D16" s="187" t="n"/>
+      <c r="E16" s="181" t="n"/>
+      <c r="F16" s="182" t="n"/>
+      <c r="G16" s="183" t="n"/>
+      <c r="H16" s="184" t="n"/>
       <c r="I16" s="182" t="n"/>
       <c r="J16" s="183" t="n"/>
       <c r="K16" s="184" t="n"/>
-      <c r="L16" s="182">
-        <f>IF(AND(AND(ISNUMBER(F16),ISNUMBER(I16),ISNUMBER(H16),ISNUMBER(K16)),F16&gt;0,I16&gt;0,H16&lt;&gt;0),ROUND(MIN(F16,I16)*(K16/I16-H16/F16),8),"")</f>
-        <v/>
-      </c>
-      <c r="M16" s="183">
-        <f>IF(AND(AND(ISNUMBER(F16),ISNUMBER(I16),ISNUMBER(H16),ISNUMBER(K16)),F16&gt;0,I16&gt;0,H16&lt;&gt;0),ROUND((K16/I16)/(H16/F16)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="L16" s="182" t="n"/>
+      <c r="M16" s="183" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="B4:M16">
@@ -2825,6 +2699,11 @@
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B5:M200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND($B5&lt;&gt;"",COUNTIF(Закрытые!$B$5:$B$200,$B5)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -2933,35 +2812,35 @@
         </is>
       </c>
       <c r="C5" s="176">
-        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5))</f>
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B5)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B5))</f>
         <v/>
       </c>
       <c r="D5" s="177">
-        <f>IF(C5="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C5)</f>
+        <f>IF(C5="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B5)*Закрытые!$G$5:$G$200*Закрытые!$H$5:$H$200))/C5)</f>
         <v/>
       </c>
       <c r="E5" s="178">
-        <f>IF(C5="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B5))</f>
+        <f>IF(C5="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B5))</f>
         <v/>
       </c>
       <c r="F5" s="176">
-        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5))</f>
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B5)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B5))</f>
         <v/>
       </c>
       <c r="G5" s="177">
-        <f>IF(F5="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F5)</f>
+        <f>IF(F5="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B5)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B5)*Закрытые!$J$5:$J$200*Закрытые!$K$5:$K$200))/F5)</f>
         <v/>
       </c>
       <c r="H5" s="178">
-        <f>IF(F5="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B5))</f>
+        <f>IF(F5="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B5)+SUMIFS(Закрытые!$L$5:$L$200,Закрытые!$F$5:$F$200,$B5))</f>
         <v/>
       </c>
       <c r="I5" s="176">
-        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND(MIN(C5,F5)*(H5/F5-E5/C5),8),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B5)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B5),8))</f>
         <v/>
       </c>
       <c r="J5" s="178">
-        <f>IF(AND(AND(ISNUMBER(C5),ISNUMBER(F5),ISNUMBER(E5),ISNUMBER(H5)),C5&gt;0,F5&gt;0,E5&lt;&gt;0),ROUND((H5/F5)/(E5/C5)*100-100,2),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B5)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B5)/SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B5)*100,2))</f>
         <v/>
       </c>
       <c r="K5" s="176" t="n"/>
@@ -2975,35 +2854,35 @@
         </is>
       </c>
       <c r="C6" s="182">
-        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6))</f>
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B6)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B6))</f>
         <v/>
       </c>
       <c r="D6" s="183">
-        <f>IF(C6="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C6)</f>
+        <f>IF(C6="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B6)*Закрытые!$G$5:$G$200*Закрытые!$H$5:$H$200))/C6)</f>
         <v/>
       </c>
       <c r="E6" s="184">
-        <f>IF(C6="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B6))</f>
+        <f>IF(C6="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B6))</f>
         <v/>
       </c>
       <c r="F6" s="182">
-        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6))</f>
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B6)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B6))</f>
         <v/>
       </c>
       <c r="G6" s="183">
-        <f>IF(F6="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F6)</f>
+        <f>IF(F6="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B6)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B6)*Закрытые!$J$5:$J$200*Закрытые!$K$5:$K$200))/F6)</f>
         <v/>
       </c>
       <c r="H6" s="184">
-        <f>IF(F6="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B6))</f>
+        <f>IF(F6="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B6)+SUMIFS(Закрытые!$L$5:$L$200,Закрытые!$F$5:$F$200,$B6))</f>
         <v/>
       </c>
       <c r="I6" s="182">
-        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND(MIN(C6,F6)*(H6/F6-E6/C6),8),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B6)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B6),8))</f>
         <v/>
       </c>
       <c r="J6" s="184">
-        <f>IF(AND(AND(ISNUMBER(C6),ISNUMBER(F6),ISNUMBER(E6),ISNUMBER(H6)),C6&gt;0,F6&gt;0,E6&lt;&gt;0),ROUND((H6/F6)/(E6/C6)*100-100,2),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B6)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B6)/SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B6)*100,2))</f>
         <v/>
       </c>
       <c r="K6" s="182" t="n"/>
@@ -3017,35 +2896,35 @@
         </is>
       </c>
       <c r="C7" s="176">
-        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7))</f>
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B7)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B7))</f>
         <v/>
       </c>
       <c r="D7" s="177">
-        <f>IF(C7="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C7)</f>
+        <f>IF(C7="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B7)*Закрытые!$G$5:$G$200*Закрытые!$H$5:$H$200))/C7)</f>
         <v/>
       </c>
       <c r="E7" s="178">
-        <f>IF(C7="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B7))</f>
+        <f>IF(C7="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B7))</f>
         <v/>
       </c>
       <c r="F7" s="176">
-        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7))</f>
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B7)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B7))</f>
         <v/>
       </c>
       <c r="G7" s="177">
-        <f>IF(F7="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F7)</f>
+        <f>IF(F7="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B7)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B7)*Закрытые!$J$5:$J$200*Закрытые!$K$5:$K$200))/F7)</f>
         <v/>
       </c>
       <c r="H7" s="178">
-        <f>IF(F7="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B7))</f>
+        <f>IF(F7="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B7)+SUMIFS(Закрытые!$L$5:$L$200,Закрытые!$F$5:$F$200,$B7))</f>
         <v/>
       </c>
       <c r="I7" s="176">
-        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND(MIN(C7,F7)*(H7/F7-E7/C7),8),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B7)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B7),8))</f>
         <v/>
       </c>
       <c r="J7" s="178">
-        <f>IF(AND(AND(ISNUMBER(C7),ISNUMBER(F7),ISNUMBER(E7),ISNUMBER(H7)),C7&gt;0,F7&gt;0,E7&lt;&gt;0),ROUND((H7/F7)/(E7/C7)*100-100,2),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B7)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B7)/SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B7)*100,2))</f>
         <v/>
       </c>
       <c r="K7" s="176" t="n"/>
@@ -3059,35 +2938,35 @@
         </is>
       </c>
       <c r="C8" s="182">
-        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8))</f>
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B8)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B8))</f>
         <v/>
       </c>
       <c r="D8" s="183">
-        <f>IF(C8="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C8)</f>
+        <f>IF(C8="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B8)*Закрытые!$G$5:$G$200*Закрытые!$H$5:$H$200))/C8)</f>
         <v/>
       </c>
       <c r="E8" s="184">
-        <f>IF(C8="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B8))</f>
+        <f>IF(C8="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B8))</f>
         <v/>
       </c>
       <c r="F8" s="182">
-        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8))</f>
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B8)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B8))</f>
         <v/>
       </c>
       <c r="G8" s="183">
-        <f>IF(F8="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F8)</f>
+        <f>IF(F8="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B8)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B8)*Закрытые!$J$5:$J$200*Закрытые!$K$5:$K$200))/F8)</f>
         <v/>
       </c>
       <c r="H8" s="184">
-        <f>IF(F8="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B8))</f>
+        <f>IF(F8="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B8)+SUMIFS(Закрытые!$L$5:$L$200,Закрытые!$F$5:$F$200,$B8))</f>
         <v/>
       </c>
       <c r="I8" s="182">
-        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND(MIN(C8,F8)*(H8/F8-E8/C8),8),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B8)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B8),8))</f>
         <v/>
       </c>
       <c r="J8" s="184">
-        <f>IF(AND(AND(ISNUMBER(C8),ISNUMBER(F8),ISNUMBER(E8),ISNUMBER(H8)),C8&gt;0,F8&gt;0,E8&lt;&gt;0),ROUND((H8/F8)/(E8/C8)*100-100,2),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B8)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B8)/SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B8)*100,2))</f>
         <v/>
       </c>
       <c r="K8" s="182" t="n"/>
@@ -3101,35 +2980,35 @@
         </is>
       </c>
       <c r="C9" s="176">
-        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9))</f>
+        <f>IF(SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B9)=0,"",SUMIFS(Торговля!$F$5:$F$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$G$5:$G$200,Закрытые!$F$5:$F$200,$B9))</f>
         <v/>
       </c>
       <c r="D9" s="177">
-        <f>IF(C9="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)/C9)</f>
+        <f>IF(C9="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$F$5:$F$200*Торговля!$G$5:$G$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B9)*Закрытые!$G$5:$G$200*Закрытые!$H$5:$H$200))/C9)</f>
         <v/>
       </c>
       <c r="E9" s="178">
-        <f>IF(C9="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B9))</f>
+        <f>IF(C9="","",SUMIFS(Торговля!$H$5:$H$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B9))</f>
         <v/>
       </c>
       <c r="F9" s="176">
-        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9))</f>
+        <f>IF(SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B9)=0,"",SUMIFS(Торговля!$I$5:$I$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$J$5:$J$200,Закрытые!$F$5:$F$200,$B9))</f>
         <v/>
       </c>
       <c r="G9" s="177">
-        <f>IF(F9="","",SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)/F9)</f>
+        <f>IF(F9="","",(SUMPRODUCT((Торговля!$E$5:$E$200=$B9)*Торговля!$I$5:$I$200*Торговля!$J$5:$J$200)+SUMPRODUCT((Закрытые!$F$5:$F$200=$B9)*Закрытые!$J$5:$J$200*Закрытые!$K$5:$K$200))/F9)</f>
         <v/>
       </c>
       <c r="H9" s="178">
-        <f>IF(F9="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B9))</f>
+        <f>IF(F9="","",SUMIFS(Торговля!$K$5:$K$200,Торговля!$E$5:$E$200,$B9)+SUMIFS(Закрытые!$L$5:$L$200,Закрытые!$F$5:$F$200,$B9))</f>
         <v/>
       </c>
       <c r="I9" s="176">
-        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND(MIN(C9,F9)*(H9/F9-E9/C9),8),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B9)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B9),8))</f>
         <v/>
       </c>
       <c r="J9" s="178">
-        <f>IF(AND(AND(ISNUMBER(C9),ISNUMBER(F9),ISNUMBER(E9),ISNUMBER(H9)),C9&gt;0,F9&gt;0,E9&lt;&gt;0),ROUND((H9/F9)/(E9/C9)*100-100,2),"")</f>
+        <f>IF(COUNTIFS(Закрытые!$F$5:$F$200,$B9)=0,"",ROUND(SUMIFS(Закрытые!$M$5:$M$200,Закрытые!$F$5:$F$200,$B9)/SUMIFS(Закрытые!$I$5:$I$200,Закрытые!$F$5:$F$200,$B9)*100,2))</f>
         <v/>
       </c>
       <c r="K9" s="176" t="n"/>
@@ -3144,14 +3023,8 @@
       <c r="F10" s="182" t="n"/>
       <c r="G10" s="183" t="n"/>
       <c r="H10" s="184" t="n"/>
-      <c r="I10" s="182">
-        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND(MIN(C10,F10)*(H10/F10-E10/C10),8),"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="184">
-        <f>IF(AND(AND(ISNUMBER(C10),ISNUMBER(F10),ISNUMBER(E10),ISNUMBER(H10)),C10&gt;0,F10&gt;0,E10&lt;&gt;0),ROUND((H10/F10)/(E10/C10)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="I10" s="182" t="n"/>
+      <c r="J10" s="184" t="n"/>
       <c r="K10" s="182" t="n"/>
       <c r="L10" s="183" t="n"/>
       <c r="M10" s="183" t="n"/>
@@ -3164,14 +3037,8 @@
       <c r="F11" s="176" t="n"/>
       <c r="G11" s="177" t="n"/>
       <c r="H11" s="178" t="n"/>
-      <c r="I11" s="176">
-        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND(MIN(C11,F11)*(H11/F11-E11/C11),8),"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="178">
-        <f>IF(AND(AND(ISNUMBER(C11),ISNUMBER(F11),ISNUMBER(E11),ISNUMBER(H11)),C11&gt;0,F11&gt;0,E11&lt;&gt;0),ROUND((H11/F11)/(E11/C11)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="I11" s="176" t="n"/>
+      <c r="J11" s="178" t="n"/>
       <c r="K11" s="176" t="n"/>
       <c r="L11" s="177" t="n"/>
       <c r="M11" s="177" t="n"/>
@@ -3184,14 +3051,8 @@
       <c r="F12" s="182" t="n"/>
       <c r="G12" s="183" t="n"/>
       <c r="H12" s="184" t="n"/>
-      <c r="I12" s="182">
-        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND(MIN(C12,F12)*(H12/F12-E12/C12),8),"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="184">
-        <f>IF(AND(AND(ISNUMBER(C12),ISNUMBER(F12),ISNUMBER(E12),ISNUMBER(H12)),C12&gt;0,F12&gt;0,E12&lt;&gt;0),ROUND((H12/F12)/(E12/C12)*100-100,2),"")</f>
-        <v/>
-      </c>
+      <c r="I12" s="182" t="n"/>
+      <c r="J12" s="184" t="n"/>
       <c r="K12" s="182" t="n"/>
       <c r="L12" s="183" t="n"/>
       <c r="M12" s="183" t="n"/>
@@ -4943,7 +4804,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="186" t="inlineStr">
         <is>
-          <t>T-0006</t>
+          <t>T-0005</t>
         </is>
       </c>
       <c r="C5" s="209" t="n">
@@ -4954,31 +4815,31 @@
       </c>
       <c r="E5" s="186" t="inlineStr">
         <is>
-          <t>OKX</t>
+          <t>Bybit</t>
         </is>
       </c>
       <c r="F5" s="175" t="inlineStr">
         <is>
-          <t>BTC/USDT</t>
+          <t>BNB/USDT</t>
         </is>
       </c>
       <c r="G5" s="176" t="n">
-        <v>0.05</v>
+        <v>2</v>
       </c>
       <c r="H5" s="177" t="n">
-        <v>62200</v>
+        <v>585</v>
       </c>
       <c r="I5" s="178" t="n">
-        <v>3103.78</v>
+        <v>1167.66</v>
       </c>
       <c r="J5" s="176" t="n">
-        <v>0.05</v>
+        <v>2</v>
       </c>
       <c r="K5" s="177" t="n">
-        <v>63000</v>
+        <v>600</v>
       </c>
       <c r="L5" s="178" t="n">
-        <v>3143.7</v>
+        <v>1197.6</v>
       </c>
       <c r="M5" s="176">
         <f>IF(AND(AND(ISNUMBER(G5),ISNUMBER(J5),ISNUMBER(I5),ISNUMBER(L5)),G5&gt;0,J5&gt;0,I5&lt;&gt;0),ROUND(MIN(G5,J5)*(L5/J5-I5/G5),8),"")</f>
@@ -4995,11 +4856,11 @@
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="187" t="inlineStr">
         <is>
-          <t>T-0003</t>
+          <t>T-0006</t>
         </is>
       </c>
       <c r="C6" s="210" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="D6" s="210" t="n">
         <v>46300</v>
@@ -5011,26 +4872,26 @@
       </c>
       <c r="F6" s="181" t="inlineStr">
         <is>
-          <t>SOL/USDT</t>
+          <t>BTC/USDT</t>
         </is>
       </c>
       <c r="G6" s="182" t="n">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="H6" s="183" t="n">
-        <v>145</v>
+        <v>62200</v>
       </c>
       <c r="I6" s="184" t="n">
-        <v>2894.2</v>
+        <v>3103.78</v>
       </c>
       <c r="J6" s="182" t="n">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="K6" s="183" t="n">
-        <v>152</v>
+        <v>63000</v>
       </c>
       <c r="L6" s="184" t="n">
-        <v>3033.92</v>
+        <v>3143.7</v>
       </c>
       <c r="M6" s="182">
         <f>IF(AND(AND(ISNUMBER(G6),ISNUMBER(J6),ISNUMBER(I6),ISNUMBER(L6)),G6&gt;0,J6&gt;0,I6&lt;&gt;0),ROUND(MIN(G6,J6)*(L6/J6-I6/G6),8),"")</f>
@@ -5045,17 +4906,45 @@
       <c r="Q6" s="183" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="186" t="n"/>
-      <c r="C7" s="209" t="n"/>
-      <c r="D7" s="209" t="n"/>
-      <c r="E7" s="186" t="n"/>
-      <c r="F7" s="175" t="n"/>
-      <c r="G7" s="176" t="n"/>
-      <c r="H7" s="177" t="n"/>
-      <c r="I7" s="178" t="n"/>
-      <c r="J7" s="176" t="n"/>
-      <c r="K7" s="177" t="n"/>
-      <c r="L7" s="178" t="n"/>
+      <c r="B7" s="186" t="inlineStr">
+        <is>
+          <t>T-0002</t>
+        </is>
+      </c>
+      <c r="C7" s="209" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D7" s="209" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E7" s="186" t="inlineStr">
+        <is>
+          <t>Bybit</t>
+        </is>
+      </c>
+      <c r="F7" s="175" t="inlineStr">
+        <is>
+          <t>ETH/USDT</t>
+        </is>
+      </c>
+      <c r="G7" s="176" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="177" t="n">
+        <v>3200</v>
+      </c>
+      <c r="I7" s="178" t="n">
+        <v>3193.6</v>
+      </c>
+      <c r="J7" s="176" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="177" t="n">
+        <v>3350</v>
+      </c>
+      <c r="L7" s="178" t="n">
+        <v>3343.3</v>
+      </c>
       <c r="M7" s="176">
         <f>IF(AND(AND(ISNUMBER(G7),ISNUMBER(J7),ISNUMBER(I7),ISNUMBER(L7)),G7&gt;0,J7&gt;0,I7&lt;&gt;0),ROUND(MIN(G7,J7)*(L7/J7-I7/G7),8),"")</f>
         <v/>
@@ -5069,17 +4958,45 @@
       <c r="Q7" s="177" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="187" t="n"/>
-      <c r="C8" s="210" t="n"/>
-      <c r="D8" s="210" t="n"/>
-      <c r="E8" s="187" t="n"/>
-      <c r="F8" s="181" t="n"/>
-      <c r="G8" s="182" t="n"/>
-      <c r="H8" s="183" t="n"/>
-      <c r="I8" s="184" t="n"/>
-      <c r="J8" s="182" t="n"/>
-      <c r="K8" s="183" t="n"/>
-      <c r="L8" s="184" t="n"/>
+      <c r="B8" s="187" t="inlineStr">
+        <is>
+          <t>T-0003</t>
+        </is>
+      </c>
+      <c r="C8" s="210" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D8" s="210" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E8" s="187" t="inlineStr">
+        <is>
+          <t>OKX</t>
+        </is>
+      </c>
+      <c r="F8" s="181" t="inlineStr">
+        <is>
+          <t>SOL/USDT</t>
+        </is>
+      </c>
+      <c r="G8" s="182" t="n">
+        <v>20</v>
+      </c>
+      <c r="H8" s="183" t="n">
+        <v>145</v>
+      </c>
+      <c r="I8" s="184" t="n">
+        <v>2894.2</v>
+      </c>
+      <c r="J8" s="182" t="n">
+        <v>20</v>
+      </c>
+      <c r="K8" s="183" t="n">
+        <v>152</v>
+      </c>
+      <c r="L8" s="184" t="n">
+        <v>3033.92</v>
+      </c>
       <c r="M8" s="182">
         <f>IF(AND(AND(ISNUMBER(G8),ISNUMBER(J8),ISNUMBER(I8),ISNUMBER(L8)),G8&gt;0,J8&gt;0,I8&lt;&gt;0),ROUND(MIN(G8,J8)*(L8/J8-I8/G8),8),"")</f>
         <v/>
@@ -5193,6 +5110,11 @@
   <mergeCells count="1">
     <mergeCell ref="B1:Q2"/>
   </mergeCells>
+  <conditionalFormatting sqref="B5:Q200">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND($B5&lt;&gt;"",COUNTIF(Торговля!$B$5:$B$200,$B5)&gt;0)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
v6: hide filter/sort buttons in menu rows except the "Пара" column
Sheets Торговля, ИТОГО Торговля, Лэндинг, ИТОГО Лэндинг, Пул, ИТОГО ПУЛ,
Закрытые, ИТОГО: autofilter kept, buttons hidden on every column except
"Пара". Ввод and Справочники unchanged. Spec updated accordingly.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tuAUF2vfAHieMmZsacm1V
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -2692,6 +2692,17 @@
     </row>
   </sheetData>
   <autoFilter ref="B4:M16">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
     <sortState ref="B5:M16">
       <sortCondition ref="E5:E16"/>
     </sortState>
@@ -3058,7 +3069,19 @@
       <c r="M12" s="183" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="B4:M12"/>
+  <autoFilter ref="B4:M12">
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>
@@ -3533,6 +3556,17 @@
     </row>
   </sheetData>
   <autoFilter ref="B4:M12">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
     <sortState ref="B5:M12">
       <sortCondition ref="E5:E12"/>
     </sortState>
@@ -3978,7 +4012,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:M12"/>
+  <autoFilter ref="B4:M12">
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>
@@ -4257,6 +4303,11 @@
     </row>
   </sheetData>
   <autoFilter ref="B4:G12">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
     <sortState ref="B5:G12">
       <sortCondition ref="E5:E12"/>
     </sortState>
@@ -4672,7 +4723,18 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:L12"/>
+  <autoFilter ref="B4:L12">
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:L2"/>
   </mergeCells>
@@ -5106,7 +5168,23 @@
       <c r="Q12" s="183" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="B4:Q12"/>
+  <autoFilter ref="B4:Q12">
+    <filterColumn colId="0" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="12" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="13" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="14" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="15" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:Q2"/>
   </mergeCells>
@@ -5553,7 +5631,19 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B4:M12"/>
+  <autoFilter ref="B4:M12">
+    <filterColumn colId="1" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="2" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="3" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="4" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="5" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="6" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="7" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="8" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="9" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="10" hiddenButton="1" showButton="0"/>
+    <filterColumn colId="11" hiddenButton="1" showButton="0"/>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
   </mergeCells>

</xml_diff>

<commit_message>
v6: drop stale sortState from autofilter on Торговля, Лэндинг, Пул
The stored "sorted by Пара" record made Excel draw a different button on
the Пара column of these three sheets. Autofilter structure is now the same
on all eight table sheets (button visible only on "Пара").

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tuAUF2vfAHieMmZsacm1V
</commit_message>
<xml_diff>
--- a/CryptoJournal_Input_Prototype_v6.xlsx
+++ b/CryptoJournal_Input_Prototype_v6.xlsx
@@ -2703,9 +2703,6 @@
     <filterColumn colId="9" hiddenButton="1" showButton="0"/>
     <filterColumn colId="10" hiddenButton="1" showButton="0"/>
     <filterColumn colId="11" hiddenButton="1" showButton="0"/>
-    <sortState ref="B5:M16">
-      <sortCondition ref="E5:E16"/>
-    </sortState>
   </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
@@ -3567,9 +3564,6 @@
     <filterColumn colId="9" hiddenButton="1" showButton="0"/>
     <filterColumn colId="10" hiddenButton="1" showButton="0"/>
     <filterColumn colId="11" hiddenButton="1" showButton="0"/>
-    <sortState ref="B5:M12">
-      <sortCondition ref="E5:E12"/>
-    </sortState>
   </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>
@@ -4308,9 +4302,6 @@
     <filterColumn colId="2" hiddenButton="1" showButton="0"/>
     <filterColumn colId="4" hiddenButton="1" showButton="0"/>
     <filterColumn colId="5" hiddenButton="1" showButton="0"/>
-    <sortState ref="B5:G12">
-      <sortCondition ref="E5:E12"/>
-    </sortState>
   </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="B1:G2"/>

</xml_diff>